<commit_message>
Value the river properly and clean up the copy
Rebuild the river, wildlife, farm and forest question from sourced
components: dry-month river flow, Shivanasamudram and Mettur power,
farms over wet and drought years, the delta, and the catchment. Charge
what Kolar's farmers lose when eastern water is piped back. Add the
dry-season view, fix the Biligundlu wording, and remove a repeated
sentence in the opening.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016H5KxzDFyejukUbATybtPZ
</commit_message>
<xml_diff>
--- a/downloads/bengaluru-water-price-model.xlsx
+++ b/downloads/bengaluru-water-price-model.xlsx
@@ -73,33 +73,39 @@
     <definedName name="bond_rate">Inputs!$C$57</definedName>
     <definedName name="ham_rate">Inputs!$C$58</definedName>
     <definedName name="ppp_equity">Inputs!$C$59</definedName>
-    <definedName name="ngt_cr_mld">Inputs!$C$60</definedName>
-    <definedName name="catchment_rs_kl">Inputs!$C$61</definedName>
-    <definedName name="basin_loss">Inputs!$C$62</definedName>
-    <definedName name="raw_oc_rs_kl">Inputs!$C$63</definedName>
-    <definedName name="lrmc_cr_mld">Inputs!$C$64</definedName>
-    <definedName name="gw_share">Inputs!$C$65</definedName>
-    <definedName name="grid_ef">Inputs!$C$66</definedName>
-    <definedName name="scc_usd">Inputs!$C$67</definedName>
-    <definedName name="fx">Inputs!$C$68</definedName>
-    <definedName name="residual_rs_kl">Inputs!$C$69</definedName>
-    <definedName name="re_share">Inputs!$C$70</definedName>
-    <definedName name="fixed_charge">Inputs!$C$71</definedName>
-    <definedName name="b1_top">Inputs!$C$72</definedName>
-    <definedName name="b1_rate">Inputs!$C$73</definedName>
-    <definedName name="b2_top">Inputs!$C$74</definedName>
-    <definedName name="b2_rate">Inputs!$C$75</definedName>
-    <definedName name="b3_top">Inputs!$C$76</definedName>
-    <definedName name="b3_rate">Inputs!$C$77</definedName>
-    <definedName name="b4_rate">Inputs!$C$78</definedName>
-    <definedName name="connections_lakh">Inputs!$C$79</definedName>
-    <definedName name="hh_size">Inputs!$C$80</definedName>
-    <definedName name="lpcd_norm">Inputs!$C$81</definedName>
-    <definedName name="hh_income_low">Inputs!$C$82</definedName>
-    <definedName name="hh_income_mid">Inputs!$C$83</definedName>
-    <definedName name="afford_pct">Inputs!$C$84</definedName>
-    <definedName name="tanker_rs_kl">Inputs!$C$85</definedName>
-    <definedName name="sanchari_rs_kl">Inputs!$C$86</definedName>
+    <definedName name="raw_oc_rs_kl">Inputs!$C$60</definedName>
+    <definedName name="ngt_cr_mld">Inputs!$C$61</definedName>
+    <definedName name="catchment_rs_kl">Inputs!$C$62</definedName>
+    <definedName name="eflow_rs_kl">Inputs!$C$63</definedName>
+    <definedName name="hydro_w_rs_kl">Inputs!$C$64</definedName>
+    <definedName name="hydro_n_rs_kl">Inputs!$C$65</definedName>
+    <definedName name="delta_rs_kl">Inputs!$C$66</definedName>
+    <definedName name="gwrech_rs_kl">Inputs!$C$67</definedName>
+    <definedName name="kolar_rs_kl">Inputs!$C$68</definedName>
+    <definedName name="basin_loss">Inputs!$C$69</definedName>
+    <definedName name="lrmc_cr_mld">Inputs!$C$70</definedName>
+    <definedName name="gw_share">Inputs!$C$71</definedName>
+    <definedName name="grid_ef">Inputs!$C$72</definedName>
+    <definedName name="scc_usd">Inputs!$C$73</definedName>
+    <definedName name="fx">Inputs!$C$74</definedName>
+    <definedName name="residual_rs_kl">Inputs!$C$75</definedName>
+    <definedName name="re_share">Inputs!$C$76</definedName>
+    <definedName name="fixed_charge">Inputs!$C$77</definedName>
+    <definedName name="b1_top">Inputs!$C$78</definedName>
+    <definedName name="b1_rate">Inputs!$C$79</definedName>
+    <definedName name="b2_top">Inputs!$C$80</definedName>
+    <definedName name="b2_rate">Inputs!$C$81</definedName>
+    <definedName name="b3_top">Inputs!$C$82</definedName>
+    <definedName name="b3_rate">Inputs!$C$83</definedName>
+    <definedName name="b4_rate">Inputs!$C$84</definedName>
+    <definedName name="connections_lakh">Inputs!$C$85</definedName>
+    <definedName name="hh_size">Inputs!$C$86</definedName>
+    <definedName name="lpcd_norm">Inputs!$C$87</definedName>
+    <definedName name="hh_income_low">Inputs!$C$88</definedName>
+    <definedName name="hh_income_mid">Inputs!$C$89</definedName>
+    <definedName name="afford_pct">Inputs!$C$90</definedName>
+    <definedName name="tanker_rs_kl">Inputs!$C$91</definedName>
+    <definedName name="sanchari_rs_kl">Inputs!$C$92</definedName>
     <definedName name="prod_kl">Ladder!$B$2</definedName>
     <definedName name="billed_kl">Ladder!$B$3</definedName>
     <definedName name="sew_kl">Ladder!$B$4</definedName>
@@ -129,21 +135,22 @@
     <definedName name="l_reserve">Ladder!$B$28</definedName>
     <definedName name="financial">Ladder!$B$29</definedName>
     <definedName name="lost">Ladder!$B$30</definedName>
-    <definedName name="l_raw">Ladder!$B$31</definedName>
-    <definedName name="l_catch">Ladder!$B$32</definedName>
-    <definedName name="economic">Ladder!$B$33</definedName>
-    <definedName name="water_kwh">Ladder!$B$34</definedName>
-    <definedName name="sew_kwh">Ladder!$B$35</definedName>
-    <definedName name="kwh_billed">Ladder!$B$36</definedName>
-    <definedName name="l_carbon">Ladder!$B$37</definedName>
-    <definedName name="l_residual">Ladder!$B$38</definedName>
-    <definedName name="social">Ladder!$B$39</definedName>
-    <definedName name="fin_deliv">Ladder!$B$40</definedName>
-    <definedName name="fin_eff">Ladder!$B$41</definedName>
-    <definedName name="regulator">Ladder!$B$42</definedName>
-    <definedName name="gap_mld">Ladder!$B$43</definedName>
-    <definedName name="today_damage">Ladder!$B$44</definedName>
-    <definedName name="rev_req">Ladder!$B$45</definedName>
+    <definedName name="l_up">Ladder!$B$31</definedName>
+    <definedName name="l_raw">Ladder!$B$32</definedName>
+    <definedName name="l_kolar">Ladder!$B$33</definedName>
+    <definedName name="economic">Ladder!$B$34</definedName>
+    <definedName name="water_kwh">Ladder!$B$35</definedName>
+    <definedName name="sew_kwh">Ladder!$B$36</definedName>
+    <definedName name="kwh_billed">Ladder!$B$37</definedName>
+    <definedName name="l_carbon">Ladder!$B$38</definedName>
+    <definedName name="l_residual">Ladder!$B$39</definedName>
+    <definedName name="social">Ladder!$B$40</definedName>
+    <definedName name="fin_deliv">Ladder!$B$41</definedName>
+    <definedName name="fin_eff">Ladder!$B$42</definedName>
+    <definedName name="regulator">Ladder!$B$43</definedName>
+    <definedName name="gap_mld">Ladder!$B$44</definedName>
+    <definedName name="today_damage">Ladder!$B$45</definedName>
+    <definedName name="rev_req">Ladder!$B$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -701,7 +708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1340,7 +1347,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Send the cleaned water back to the Cauvery</t>
+          <t>Pipe the eastern valleys' cleaned water back to the Cauvery</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
@@ -2847,31 +2854,31 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ngt_cr_mld</t>
+          <t>raw_oc_rs_kl</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>NGT environmental compensation for untreated sewage</t>
+          <t>Downstream farming, averaged over wet and drought years</t>
         </is>
       </c>
       <c r="C60" s="4" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D60" t="n">
-        <v>2</v>
+        <v>0.9</v>
       </c>
       <c r="E60" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>₹ cr per MLD of gap</t>
+          <t>₹/kL not returned</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2883,31 +2890,31 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>catchment_rs_kl</t>
+          <t>ngt_cr_mld</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Keeping the Cauvery catchment working</t>
+          <t>NGT environmental compensation for untreated sewage</t>
         </is>
       </c>
       <c r="C61" s="4" t="n">
         <v>2</v>
       </c>
       <c r="D61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E61" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>₹/kL drawn</t>
+          <t>₹ cr per MLD of gap</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>assumed</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2919,26 +2926,26 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>basin_loss</t>
+          <t>catchment_rs_kl</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Share of the city's sewage that drains out of the Cauvery basin</t>
+          <t>Bengaluru's share of keeping the catchment forested</t>
         </is>
       </c>
       <c r="C62" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E62" t="n">
-        <v>0.7</v>
+        <v>6</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>₹/kL drawn</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2955,22 +2962,22 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>raw_oc_rs_kl</t>
+          <t>eflow_rs_kl</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Value of Cauvery water to downstream farms</t>
+          <t>River flow for fish and wildlife in the dry months</t>
         </is>
       </c>
       <c r="C63" s="4" t="n">
         <v>4</v>
       </c>
       <c r="D63" t="n">
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="E63" t="n">
-        <v>11</v>
+        <v>7.3</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -2984,33 +2991,33 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Scarcity and the river</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>lrmc_cr_mld</t>
+          <t>hydro_w_rs_kl</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Cost of the next source (Stage VI: ₹6,939 cr / 500 MLD)</t>
+          <t>Hydropower lost at Shivanasamudram</t>
         </is>
       </c>
       <c r="C64" s="4" t="n">
-        <v>13.9</v>
+        <v>0.57</v>
       </c>
       <c r="D64" t="n">
-        <v>10.3</v>
+        <v>0.35</v>
       </c>
       <c r="E64" t="n">
-        <v>16</v>
+        <v>1.66</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>₹ cr/MLD</t>
+          <t>₹/kL drawn</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3020,429 +3027,429 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Scarcity and the river</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>gw_share</t>
+          <t>hydro_n_rs_kl</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Share of city demand met by groundwater</t>
+          <t>Hydropower lost at Mettur and the Tamil Nadu barrages</t>
         </is>
       </c>
       <c r="C65" s="4" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="D65" t="n">
         <v>0.4</v>
       </c>
-      <c r="D65" t="n">
-        <v>0.15</v>
-      </c>
       <c r="E65" t="n">
-        <v>0.52</v>
+        <v>1.62</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>₹/kL not returned</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Scarcity and the river</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>grid_ef</t>
+          <t>delta_rs_kl</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Grid emission factor (CEA v22, FY26)</t>
+          <t>Delta and coast: seawater intrusion, mangroves</t>
         </is>
       </c>
       <c r="C66" s="4" t="n">
-        <v>0.675</v>
+        <v>0.3</v>
       </c>
       <c r="D66" t="n">
-        <v>0.512</v>
+        <v>0</v>
       </c>
       <c r="E66" t="n">
-        <v>0.727</v>
+        <v>1.5</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>tCO₂/MWh</t>
+          <t>₹/kL not returned</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>assumed</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Carbon</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>scc_usd</t>
+          <t>gwrech_rs_kl</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Social cost of carbon</t>
+          <t>Groundwater recharge downstream</t>
         </is>
       </c>
       <c r="C67" s="4" t="n">
-        <v>255</v>
+        <v>0.12</v>
       </c>
       <c r="D67" t="n">
-        <v>40</v>
+        <v>0.03</v>
       </c>
       <c r="E67" t="n">
-        <v>425</v>
+        <v>0.4</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>$/tCO₂</t>
+          <t>₹/kL not returned</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Carbon</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>fx</t>
+          <t>kolar_rs_kl</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Exchange rate (FBIL, 30 Oct 2026)</t>
+          <t>Value of treated water to Kolar and Chikkaballapur farmers</t>
         </is>
       </c>
       <c r="C68" s="4" t="n">
-        <v>95.25</v>
+        <v>15</v>
       </c>
       <c r="D68" t="n">
-        <v>94.40000000000001</v>
+        <v>5</v>
       </c>
       <c r="E68" t="n">
-        <v>96.8</v>
+        <v>30</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>₹/$</t>
+          <t>₹/kL</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Carbon</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>residual_rs_kl</t>
+          <t>basin_loss</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Residual harm after treating sewage to NGT norms</t>
+          <t>Share of the city's sewage that drains out of the Cauvery basin</t>
         </is>
       </c>
       <c r="C69" s="4" t="n">
-        <v>8</v>
+        <v>0.6</v>
       </c>
       <c r="D69" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="E69" t="n">
-        <v>12</v>
+        <v>0.7</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>₹/kL sewage</t>
+          <t>share</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>assumed</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Climate and residual harm</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>re_share</t>
+          <t>lrmc_cr_mld</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Share of BWSSB power bought from renewables</t>
+          <t>Cost of the next source (Stage VI: ₹6,939 cr / 500 MLD)</t>
         </is>
       </c>
       <c r="C70" s="4" t="n">
-        <v>0</v>
+        <v>13.9</v>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>10.3</v>
       </c>
       <c r="E70" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>₹ cr/MLD</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Climate and residual harm</t>
+          <t>Scarcity and the river</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>fixed_charge</t>
+          <t>gw_share</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Fixed charge per connection</t>
+          <t>Share of city demand met by groundwater</t>
         </is>
       </c>
       <c r="C71" s="4" t="n">
-        <v>100</v>
+        <v>0.4</v>
       </c>
       <c r="D71" t="n">
-        <v>50</v>
+        <v>0.15</v>
       </c>
       <c r="E71" t="n">
-        <v>150</v>
+        <v>0.52</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>₹/connection/month</t>
+          <t>share</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Scarcity and the river</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>b1_top</t>
+          <t>grid_ef</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Lifeline block: upper limit</t>
+          <t>Grid emission factor (CEA v22, FY26)</t>
         </is>
       </c>
       <c r="C72" s="4" t="n">
-        <v>10</v>
+        <v>0.675</v>
       </c>
       <c r="D72" t="n">
-        <v>8</v>
+        <v>0.512</v>
       </c>
       <c r="E72" t="n">
-        <v>15</v>
+        <v>0.727</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>kL/month</t>
+          <t>tCO₂/MWh</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Carbon</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>b1_rate</t>
+          <t>scc_usd</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Lifeline block: rate (all-in)</t>
+          <t>Social cost of carbon</t>
         </is>
       </c>
       <c r="C73" s="4" t="n">
-        <v>15</v>
+        <v>255</v>
       </c>
       <c r="D73" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="E73" t="n">
-        <v>25</v>
+        <v>425</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>₹/kL</t>
+          <t>$/tCO₂</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Carbon</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>b2_top</t>
+          <t>fx</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Second block: upper limit</t>
+          <t>Exchange rate (FBIL, 30 Oct 2026)</t>
         </is>
       </c>
       <c r="C74" s="4" t="n">
-        <v>20</v>
+        <v>95.25</v>
       </c>
       <c r="D74" t="n">
-        <v>15</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="E74" t="n">
-        <v>30</v>
+        <v>96.8</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>kL/month</t>
+          <t>₹/$</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Carbon</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>b2_rate</t>
+          <t>residual_rs_kl</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Second block: rate</t>
+          <t>Residual harm after treating sewage to NGT norms</t>
         </is>
       </c>
       <c r="C75" s="4" t="n">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="D75" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="E75" t="n">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>₹/kL</t>
+          <t>₹/kL sewage</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Climate and residual harm</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>b3_top</t>
+          <t>re_share</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Third block: upper limit</t>
+          <t>Share of BWSSB power bought from renewables</t>
         </is>
       </c>
       <c r="C76" s="4" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D76" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E76" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>kL/month</t>
+          <t>share</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3452,33 +3459,33 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Climate and residual harm</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>b3_rate</t>
+          <t>fixed_charge</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Third block: rate</t>
+          <t>Fixed charge per connection</t>
         </is>
       </c>
       <c r="C77" s="4" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="D77" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="E77" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>₹/kL</t>
+          <t>₹/connection/month</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3495,26 +3502,26 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>b4_rate</t>
+          <t>b1_top</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Top block: rate</t>
+          <t>Lifeline block: upper limit</t>
         </is>
       </c>
       <c r="C78" s="4" t="n">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="D78" t="n">
-        <v>110</v>
+        <v>8</v>
       </c>
       <c r="E78" t="n">
-        <v>220</v>
+        <v>15</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>₹/kL</t>
+          <t>kL/month</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3531,31 +3538,31 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>connections_lakh</t>
+          <t>b1_rate</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Water connections</t>
+          <t>Lifeline block: rate (all-in)</t>
         </is>
       </c>
       <c r="C79" s="4" t="n">
-        <v>11.3</v>
+        <v>15</v>
       </c>
       <c r="D79" t="n">
-        <v>10.7</v>
+        <v>8</v>
       </c>
       <c r="E79" t="n">
-        <v>11.5</v>
+        <v>25</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>lakh</t>
+          <t>₹/kL</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3567,250 +3574,466 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>hh_size</t>
+          <t>b2_top</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Persons per household, Bengaluru</t>
+          <t>Second block: upper limit</t>
         </is>
       </c>
       <c r="C80" s="4" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D80" t="n">
-        <v>3.5</v>
+        <v>15</v>
       </c>
       <c r="E80" t="n">
-        <v>4.5</v>
+        <v>30</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>persons</t>
+          <t>kL/month</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>lpcd_norm</t>
+          <t>b2_rate</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Water each person needs (CPHEEO norm)</t>
+          <t>Second block: rate</t>
         </is>
       </c>
       <c r="C81" s="4" t="n">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="D81" t="n">
-        <v>108</v>
+        <v>40</v>
       </c>
       <c r="E81" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>litres/person/day</t>
+          <t>₹/kL</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>hh_income_low</t>
+          <t>b3_top</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Lower-income household income</t>
+          <t>Third block: upper limit</t>
         </is>
       </c>
       <c r="C82" s="4" t="n">
-        <v>25000</v>
+        <v>40</v>
       </c>
       <c r="D82" t="n">
-        <v>15000</v>
+        <v>30</v>
       </c>
       <c r="E82" t="n">
-        <v>35000</v>
+        <v>60</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>₹/month</t>
+          <t>kL/month</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>assumed</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>hh_income_mid</t>
+          <t>b3_rate</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Middle-income household income</t>
+          <t>Third block: rate</t>
         </is>
       </c>
       <c r="C83" s="4" t="n">
-        <v>75000</v>
+        <v>105</v>
       </c>
       <c r="D83" t="n">
-        <v>42000</v>
+        <v>90</v>
       </c>
       <c r="E83" t="n">
-        <v>125000</v>
+        <v>130</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>₹/month</t>
+          <t>₹/kL</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>assumed</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>afford_pct</t>
+          <t>b4_rate</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Affordability threshold (share of income)</t>
+          <t>Top block: rate</t>
         </is>
       </c>
       <c r="C84" s="4" t="n">
-        <v>0.03</v>
+        <v>150</v>
       </c>
       <c r="D84" t="n">
-        <v>0.03</v>
+        <v>110</v>
       </c>
       <c r="E84" t="n">
-        <v>0.05</v>
+        <v>220</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>share of income</t>
+          <t>₹/kL</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>tanker_rs_kl</t>
+          <t>connections_lakh</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Private tanker water price (2025-26)</t>
+          <t>Water connections</t>
         </is>
       </c>
       <c r="C85" s="4" t="n">
-        <v>140</v>
+        <v>11.3</v>
       </c>
       <c r="D85" t="n">
-        <v>115</v>
+        <v>10.7</v>
       </c>
       <c r="E85" t="n">
-        <v>210</v>
+        <v>11.5</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>₹/kL</t>
+          <t>lakh</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>hh_size</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Persons per household, Bengaluru</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D86" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E86" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>lpcd_norm</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Water each person needs (CPHEEO norm)</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="n">
+        <v>135</v>
+      </c>
+      <c r="D87" t="n">
+        <v>108</v>
+      </c>
+      <c r="E87" t="n">
+        <v>150</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>litres/person/day</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>hh_income_low</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Lower-income household income</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D88" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E88" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>₹/month</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>hh_income_mid</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Middle-income household income</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="n">
+        <v>75000</v>
+      </c>
+      <c r="D89" t="n">
+        <v>42000</v>
+      </c>
+      <c r="E89" t="n">
+        <v>125000</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>₹/month</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>afford_pct</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Affordability threshold (share of income)</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D90" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>share of income</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>tanker_rs_kl</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Private tanker water price (2025-26)</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="D91" t="n">
+        <v>115</v>
+      </c>
+      <c r="E91" t="n">
+        <v>210</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>₹/kL</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
           <t>sanchari_rs_kl</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>BWSSB Sanchari Cauvery tanker price</t>
         </is>
       </c>
-      <c r="C86" s="4" t="n">
+      <c r="C92" s="4" t="n">
         <v>108</v>
       </c>
-      <c r="D86" t="n">
+      <c r="D92" t="n">
         <v>107</v>
       </c>
-      <c r="E86" t="n">
+      <c r="E92" t="n">
         <v>165</v>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F92" t="inlineStr">
         <is>
           <t>₹/kL</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
+      <c r="G92" t="inlineStr">
         <is>
           <t>reference</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H92" t="inlineStr">
         <is>
           <t>Households and affordability</t>
         </is>
@@ -3827,7 +4050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -4243,12 +4466,12 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>return_on*polish_rs_kl*return_factor</f>
+        <f>polish_rs_kl*return_factor</f>
         <v/>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>return_on*polish_rs_kl*return_factor</t>
+          <t>polish_rs_kl*return_factor</t>
         </is>
       </c>
     </row>
@@ -4319,238 +4542,254 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Q7. Water for downstream farms</t>
+          <t>Q7. Lost at the intake: dry-month flow in the gorge (60%), Shivanasamudram power, catchment</t>
         </is>
       </c>
       <c r="B31" s="5">
-        <f>raw_oc_rs_kl*lost/(1-nrw)</f>
+        <f>(0.6*eflow_rs_kl+hydro_w_rs_kl+catchment_rs_kl)/(1-nrw)</f>
         <v/>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>raw_oc_rs_kl*lost/(1-nrw)</t>
+          <t>(0.6*eflow_rs_kl+hydro_w_rs_kl+catchment_rs_kl)/(1-nrw)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Q7. Catchment upkeep</t>
+          <t>Q7. Lost downstream: farms, Mettur power, delta, wells, river below Sangama</t>
         </is>
       </c>
       <c r="B32" s="5">
-        <f>catchment_rs_kl/(1-nrw)</f>
+        <f>(raw_oc_rs_kl+hydro_n_rs_kl+delta_rs_kl+gwrech_rs_kl+0.4*eflow_rs_kl)*lost/(1-nrw)</f>
         <v/>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>catchment_rs_kl/(1-nrw)</t>
+          <t>(raw_oc_rs_kl+hydro_n_rs_kl+delta_rs_kl+gwrech_rs_kl+0.4*eflow_rs_kl)*lost/(1-nrw)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Q7. What Kolar loses if the water is piped back</t>
+        </is>
+      </c>
+      <c r="B33" s="5">
+        <f>return_on*basin_loss*return_factor*kolar_rs_kl</f>
+        <v/>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>return_on*basin_loss*return_factor*kolar_rs_kl</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>RUNG 3. Full economic cost</t>
         </is>
       </c>
-      <c r="B33" s="7">
-        <f>financial+l_raw+l_catch</f>
-        <v/>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>financial+l_raw+l_catch</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Water-side electricity, kWh/yr</t>
-        </is>
-      </c>
-      <c r="B34" s="5">
-        <f>(energy_m-sew_energy_cr_m*prod_scale)*12*1E7/electricity_rs_kwh</f>
+      <c r="B34" s="7">
+        <f>financial+l_up+l_raw+l_kolar</f>
         <v/>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>(energy_m-sew_energy_cr_m*prod_scale)*12*1E7/electricity_rs_kwh</t>
+          <t>financial+l_up+l_raw+l_kolar</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sewerage electricity per kL sewage</t>
+          <t>Water-side electricity, kWh/yr</t>
         </is>
       </c>
       <c r="B35" s="5">
-        <f>sew_energy_cr_m*12*1E7/electricity_rs_kwh/treated_kl</f>
+        <f>(energy_m-sew_energy_cr_m*prod_scale)*12*1E7/electricity_rs_kwh</f>
         <v/>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>sew_energy_cr_m*12*1E7/electricity_rs_kwh/treated_kl</t>
+          <t>(energy_m-sew_energy_cr_m*prod_scale)*12*1E7/electricity_rs_kwh</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>kWh per kL billed</t>
+          <t>Sewerage electricity per kL sewage</t>
         </is>
       </c>
       <c r="B36" s="5">
-        <f>water_kwh/billed_kl+sew_kwh*return_factor+return_on*basin_loss*return_factor*ret_kwh</f>
+        <f>sew_energy_cr_m*12*1E7/electricity_rs_kwh/treated_kl</f>
         <v/>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>water_kwh/billed_kl+sew_kwh*return_factor+return_on*basin_loss*return_factor*ret_kwh</t>
+          <t>sew_energy_cr_m*12*1E7/electricity_rs_kwh/treated_kl</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Q8. Carbon</t>
+          <t>kWh per kL billed</t>
         </is>
       </c>
       <c r="B37" s="5">
-        <f>kwh_billed*grid_ef*(1-re_share)/1000*scc_usd*fx</f>
+        <f>water_kwh/billed_kl+sew_kwh*return_factor+return_on*basin_loss*return_factor*ret_kwh</f>
         <v/>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>kwh_billed*grid_ef*(1-re_share)/1000*scc_usd*fx</t>
+          <t>water_kwh/billed_kl+sew_kwh*return_factor+return_on*basin_loss*return_factor*ret_kwh</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>Q8. Carbon</t>
+        </is>
+      </c>
+      <c r="B38" s="5">
+        <f>kwh_billed*grid_ef*(1-re_share)/1000*scc_usd*fx</f>
+        <v/>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>kwh_billed*grid_ef*(1-re_share)/1000*scc_usd*fx</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Q8. Residual harm after treatment</t>
         </is>
       </c>
-      <c r="B38" s="5">
+      <c r="B39" s="5">
         <f>residual_rs_kl*return_factor</f>
         <v/>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>residual_rs_kl*return_factor</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>RUNG 4. Full social cost</t>
         </is>
       </c>
-      <c r="B39" s="7">
+      <c r="B40" s="7">
         <f>economic+l_carbon+l_residual</f>
         <v/>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Rogers et al.: full cost</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Per kL delivered (incl. unbilled use)</t>
-        </is>
-      </c>
-      <c r="B40" s="5">
-        <f>financial*billed_kl/(prod_kl*(1-nrw*nrw_phys_share))</f>
-        <v/>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>financial*billed_kl/(prod_kl*(1-nrw*nrw_phys_share))</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>At efficient losses</t>
+          <t>Per kL delivered (incl. unbilled use)</t>
         </is>
       </c>
       <c r="B41" s="5">
-        <f>financial*(1-nrw)/(1-MIN(nrw,nrw_efficient))</f>
+        <f>financial*billed_kl/(prod_kl*(1-nrw*nrw_phys_share))</f>
         <v/>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>financial*(1-nrw)/(1-MIN(nrw,nrw_efficient))</t>
+          <t>financial*billed_kl/(prod_kl*(1-nrw*nrw_phys_share))</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Regulator's view on historical books</t>
+          <t>At efficient losses</t>
         </is>
       </c>
       <c r="B42" s="5">
-        <f>(opex_m*12*1E7+rab_hist_cr*1E7*(reg_dep+reg_wacc_nom))/billed_kl</f>
+        <f>financial*(1-nrw)/(1-MIN(nrw,nrw_efficient))</f>
         <v/>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>(opex_m*12*1E7+rab_hist_cr*1E7*(reg_dep+reg_wacc_nom))/billed_kl</t>
+          <t>financial*(1-nrw)/(1-MIN(nrw,nrw_efficient))</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Untreated sewage, MLD</t>
+          <t>Regulator's view on historical books</t>
         </is>
       </c>
       <c r="B43" s="5">
-        <f>MAX(0,sewage_mld-treated_mld-decentral_mld)</f>
+        <f>(opex_m*12*1E7+rab_hist_cr*1E7*(reg_dep+reg_wacc_nom))/billed_kl</f>
         <v/>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MAX(0,sewage_mld-treated_mld-decentral_mld)</t>
+          <t>(opex_m*12*1E7+rab_hist_cr*1E7*(reg_dep+reg_wacc_nom))/billed_kl</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Today's untreated-sewage damage (not in price)</t>
+          <t>Untreated sewage, MLD</t>
         </is>
       </c>
       <c r="B44" s="5">
-        <f>gap_mld*ngt_cr_mld*1E7/billed_kl</f>
+        <f>MAX(0,sewage_mld-treated_mld-decentral_mld)</f>
         <v/>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>NGT rate read as one year of damage</t>
+          <t>MAX(0,sewage_mld-treated_mld-decentral_mld)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>Today's untreated-sewage damage (not in price)</t>
+        </is>
+      </c>
+      <c r="B45" s="5">
+        <f>gap_mld*ngt_cr_mld*1E7/billed_kl</f>
+        <v/>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>NGT rate read as one year of damage</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>Revenue needed at rung 2, ₹ cr/yr</t>
         </is>
       </c>
-      <c r="B45" s="5">
+      <c r="B46" s="5">
         <f>financial*billed_kl/1E7</f>
         <v/>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>financial*billed_kl/1E7</t>
         </is>
@@ -7242,10 +7481,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>58.1</v>
+        <v>57.9</v>
       </c>
       <c r="C4" t="n">
-        <v>67.59999999999999</v>
+        <v>67.7</v>
       </c>
     </row>
     <row r="5">
@@ -7255,10 +7494,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>107.9</v>
+        <v>107.3</v>
       </c>
       <c r="C5" t="n">
-        <v>128.9</v>
+        <v>128.8</v>
       </c>
     </row>
     <row r="6">
@@ -7268,10 +7507,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>115.4</v>
+        <v>126.3</v>
       </c>
       <c r="C6" t="n">
-        <v>137.1</v>
+        <v>150.6</v>
       </c>
     </row>
     <row r="7">
@@ -7281,10 +7520,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>164.3</v>
+        <v>175.3</v>
       </c>
       <c r="C7" t="n">
-        <v>228.3</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10">
@@ -7631,10 +7870,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>-7.3</v>
+        <v>-7.5</v>
       </c>
       <c r="D29" t="n">
-        <v>25.5</v>
+        <v>26.2</v>
       </c>
     </row>
     <row r="30">
@@ -7712,163 +7951,163 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>dist_cr_km</t>
+          <t>kolar_rs_kl</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Replacement cost of distribution, incl. reservoirs</t>
+          <t>Value of treated water to Kolar and Chikkaballapur farmers</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>-3</v>
+        <v>-4.8</v>
       </c>
       <c r="D34" t="n">
-        <v>6.1</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>energy_cr_m</t>
+          <t>dist_cr_km</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>of which electricity</t>
+          <t>Replacement cost of distribution, incl. reservoirs</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>-5.3</v>
+        <v>-3</v>
       </c>
       <c r="D35" t="n">
-        <v>3.5</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>catchment_rs_kl</t>
+          <t>return_factor</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Keeping the Cauvery catchment working (NYC spends ~₹7/kL on its watershed)</t>
+          <t>Sewage returned per kL of water used</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>-1.4</v>
+        <v>-6</v>
       </c>
       <c r="D36" t="n">
-        <v>7.1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>bulk_cr_mld</t>
+          <t>energy_cr_m</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Replacement cost of bulk supply (Stage V ≈ 5.6-7.1)</t>
+          <t>of which electricity</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>-3.3</v>
+        <v>-5.3</v>
       </c>
       <c r="D37" t="n">
-        <v>4.8</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>return_factor</t>
+          <t>bulk_cr_mld</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Sewage returned per kL of water used</t>
+          <t>Replacement cost of bulk supply (Stage V ≈ 5.6-7.1)</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>-5.3</v>
+        <v>-3.3</v>
       </c>
       <c r="D38" t="n">
-        <v>2.6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>life_bulk</t>
+          <t>catchment_rs_kl</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Life: bulk and distribution</t>
+          <t>Bengaluru's share of keeping the catchment forested</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>4.1</v>
+        <v>-0.9</v>
       </c>
       <c r="D39" t="n">
-        <v>-3.6</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>opex_cr_m</t>
+          <t>life_bulk</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BWSSB operating spend (Aug 2025)</t>
+          <t>Life: bulk and distribution</t>
         </is>
       </c>
       <c r="C40" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="D40" t="n">
         <v>-3.6</v>
-      </c>
-      <c r="D40" t="n">
-        <v>3.9</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>residual_rs_kl</t>
+          <t>opex_cr_m</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Residual harm after treatment: N₂O, STP methane, nutrients left at NGT limits, sludge</t>
+          <t>BWSSB operating spend (Aug 2025)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>-4</v>
+        <v>-3.6</v>
       </c>
       <c r="D41" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>polish_rs_kl</t>
+          <t>residual_rs_kl</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Extra cleaning to river quality, beyond NGT norms</t>
+          <t>Residual harm after treatment: N₂O, STP methane, nutrients left at NGT limits, sludge</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>-2.5</v>
+        <v>-4</v>
       </c>
       <c r="D42" t="n">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
     </row>
   </sheetData>
@@ -7882,7 +8121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N86"/>
+  <dimension ref="A1:N92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8979,7 +9218,7 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Send the cleaned water back to the Cauvery</t>
+          <t>Pipe the eastern valleys' cleaned water back to the Cauvery</t>
         </is>
       </c>
       <c r="D18" s="11" t="n">
@@ -9003,7 +9242,7 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>The premise of this page is that a city should give its river back the water it borrows, cleaned. Today the eastern valleys' water goes to Kolar's tanks and the South Pennar instead. Switch this off to see the price without the return pipelines.</t>
+          <t>The premise of this page is that a city should give its river back the water it borrows, cleaned. Today the eastern valleys' water goes to Kolar's tanks and the South Pennar instead. Switch this off to see the price without the return pipelines. Question 7 counts what Kolar's farmers lose when it is on.</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
@@ -11527,7 +11766,7 @@
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>ngt_cr_mld</t>
+          <t>raw_oc_rs_kl</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
@@ -11537,63 +11776,58 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>NGT environmental compensation for untreated sewage</t>
+          <t>Downstream farming, averaged over wet and drought years</t>
         </is>
       </c>
       <c r="D60" s="11" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E60" s="11" t="n">
-        <v>2</v>
+        <v>0.9</v>
       </c>
       <c r="F60" s="11" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>₹ cr per MLD of gap</t>
+          <t>₹/kL not returned</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>The National Green Tribunal fined states ₹2 crore for every million litres a day of sewage they fail to treat. In October 2022 it applied this to Karnataka's 1,427 MLD gap, giving ₹2,856 crore.</t>
+          <t>In about half the years since 1985 the Cauvery met Tamil Nadu's full share and spilled the rest to sea; then an extra kL grows nothing. In drought years like 2023-24 (delta paddy down about 40%) a kL was worth ₹7–11. Weighting wet, normal and drought years gives about ₹2–3. In a drought year the kL lost is usually Mandya sugarcane (₹4.5–5.9/kL net), because Bengaluru's water comes out of Karnataka's share.</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr">
         <is>
-          <t>The rate is a one-off compensation for past failure; the NGT did not say what period it covers. The model treats it as one year of damage (₹2 cr / 365,000 kL ≈ ₹55 per kL untreated), which is an interpretation. CPCB's separate formula builds compensation from STP capital (₹1.75 cr/MLD) plus conveyance (₹5.55 cr/MLD) plus 10% O&amp;M.</t>
+          <t>The range runs to ₹11 to show a drought year.</t>
         </is>
       </c>
       <c r="K60" s="11" t="inlineStr">
         <is>
-          <t>NGT imposes environmental compensation of Rs 2,900 cr on K'taka (DTNext / ANI, 2022): Order of 13 Oct 2022 (OA 606/2018): sewage treatment gap 1,427.4 MLD; 'compensation works out to Rs. 2856/- crores' https://www.dtnext.in/news/national/ngt-imposes-environmental-compensation-of-rs-2900-cr-on-ktaka</t>
+          <t>Price policy for kharif crops 2025-26 (CACP, 2025): Paddy costs and returns per hectare by state https://cacp.da.gov.in/Document/EnglishReports/KharifReports2025-26_20250825125215821.pdf</t>
         </is>
       </c>
       <c r="L60" s="11" t="inlineStr">
         <is>
-          <t>NGT has imposed a fine of about 80,000 crore so far on states (Down To Earth, 2023): Fine fixed at Rs 2 crore per MLD for liquid waste and Rs 300 per tonne of solid waste; Karnataka ₹3,400 cr https://www.downtoearth.org.in/waste/ngt-has-imposed-a-fine-of-about-80-000-crore-so-far-on-states-for-not-disposing-of-sewage-and-garbage-90449</t>
+          <t>Paucity of water hits harvest, paddy yield down 40% in delta (New Indian Express, 2024): 2023-24 delta paddy yield down about 40% for lack of Cauvery water https://www.newindianexpress.com/states/tamil-nadu/2024/Feb/15/tamil-nadu-paucity-of-water-hits-harvest-paddy-yield-down-40-in-delta</t>
         </is>
       </c>
       <c r="M60" s="11" t="inlineStr">
         <is>
-          <t>Compliance of MSW Rules (OA 606/2018), order of 19 May 2023 (NGT via Indian Kanoon, 2023): Compensation 'on the scale of Rs. 2 crore per MLD for gap in respect of liquid waste'; 'worked out in the light of scientific studies and cost of remediation' https://indiankanoon.org/doc/5883219</t>
-        </is>
-      </c>
-      <c r="N60" s="11" t="inlineStr">
-        <is>
-          <t>NGT Central Zone order (CPCB environmental compensation method) (NGT, 2024): CPCB method assumes STP capital ₹1.75 cr/MLD, conveyance ₹5.55 cr/MLD and annual O&amp;M at 10% of combined capital https://www.greentribunal.gov.in/gen_pdf_test.php?filepath=L25ndF9kb2N1bWVudHMvbmd0L2Nhc2Vkb2MvanVkZ2VtZW50cy9CSE9QQUwvMjAyNC0wNC0wOC8xNzEyNTY5NzY1Njg4MjQ2NTE2NjYxM2JkYTU3MWVmYy5wZGY%3D</t>
+          <t>Poor monsoon and no Cauvery water: distress in delta (The Hindu, 2026): 2026 kuruvai distress in the delta https://www.thehindu.com/news/national/tamil-nadu/poor-monsoon-and-no-cauvery-water-distress-in-delta-region-of-tamil-nadu-2026-kharif-season/article71211621.ece</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
         <is>
-          <t>catchment_rs_kl</t>
+          <t>ngt_cr_mld</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
@@ -11603,63 +11837,63 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Keeping the Cauvery catchment working</t>
+          <t>NGT environmental compensation for untreated sewage</t>
         </is>
       </c>
       <c r="D61" s="11" t="n">
         <v>2</v>
       </c>
       <c r="E61" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" s="11" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G61" s="11" t="inlineStr">
         <is>
-          <t>₹/kL drawn</t>
+          <t>₹ cr per MLD of gap</t>
         </is>
       </c>
       <c r="H61" s="11" t="inlineStr">
         <is>
-          <t>assumed</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="I61" s="11" t="inlineStr">
         <is>
-          <t>Cities that protect the land their water comes from pay for it: Quito sets aside 2% of its water utility's budget, and New York spends about ₹6-7 per kilolitre. Bengaluru pays nothing today, so ₹2 is a modest middle.</t>
+          <t>The National Green Tribunal fined states ₹2 crore for every million litres a day of sewage they fail to treat. In October 2022 it applied this to Karnataka's 1,427 MLD gap, giving ₹2,856 crore.</t>
         </is>
       </c>
       <c r="J61" s="11" t="inlineStr">
         <is>
-          <t>Arithmetic: NYC $2.9 bn over ~32 years (since 1993) ≈ $91 m/yr ÷ (1,006 MGD × 3,785 m³ × 365 = 1.39 bn m³) ≈ $0.065/m³ ≈ ₹6.2/kL (₹7.1 if counted from 1997). Quito-style 2% of BWSSB opex: ₹2,873 cr × 2% = ₹57 cr ÷ 693.5 Mm³ (1,900 MLD) ≈ ₹0.8/kL. Cauvery Calling: 242 crore trees × ₹42 = ₹10,164 cr; if Bengaluru alone paid it over 20 years ≈ ₹7.3/kL. NYC's spending avoided a filtration plant 'that could cost $10 billion or more' (DEP 2010). No study values the KRS catchment specifically.</t>
+          <t>The rate is a one-off compensation for past failure; the NGT did not say what period it covers. The model treats it as one year of damage (₹2 cr / 365,000 kL ≈ ₹55 per kL untreated), which is an interpretation. CPCB's separate formula builds compensation from STP capital (₹1.75 cr/MLD) plus conveyance (₹5.55 cr/MLD) plus 10% O&amp;M.</t>
         </is>
       </c>
       <c r="K61" s="11" t="inlineStr">
         <is>
-          <t>Filtration Avoidance Annual Report 2024 (NYC DEP, 2025): 'DEP has spent or committed more than $2.9 billion' on watershed programmes https://www.nyc.gov/assets/dep/downloads/pdf/about/filtration-avoidance-determination/2024_fad_annual.pdf</t>
+          <t>NGT imposes environmental compensation of Rs 2,900 cr on K'taka (DTNext / ANI, 2022): Order of 13 Oct 2022 (OA 606/2018): sewage treatment gap 1,427.4 MLD; 'compensation works out to Rs. 2856/- crores' https://www.dtnext.in/news/national/ngt-imposes-environmental-compensation-of-rs-2900-cr-on-ktaka</t>
         </is>
       </c>
       <c r="L61" s="11" t="inlineStr">
         <is>
-          <t>Mayor's Management Report FY2026: Department of Environmental Protection (City of New York, 2026): Average daily in-City water consumption 1,006 million gallons (FY26) https://www.nyc.gov/assets/operations/downloads/pdf/mmr2026/dep.pdf</t>
+          <t>NGT has imposed a fine of about 80,000 crore so far on states (Down To Earth, 2023): Fine fixed at Rs 2 crore per MLD for liquid waste and Rs 300 per tonne of solid waste; Karnataka ₹3,400 cr https://www.downtoearth.org.in/waste/ngt-has-imposed-a-fine-of-about-80-000-crore-so-far-on-states-for-not-disposing-of-sewage-and-garbage-90449</t>
         </is>
       </c>
       <c r="M61" s="11" t="inlineStr">
         <is>
-          <t>Water Funds: conserving green infrastructure for source water protection (Land Conservation Network / TNC, 2022): FONAG: annual budget about US$2 million; Quito's water company 'is required to contribute two percent of the water company's annual budget' (87% of funding) https://landconservationnetwork.org/wp-content/uploads/2022/08/Water20Funds_Updated_0303222028229-1.pdf</t>
+          <t>Compliance of MSW Rules (OA 606/2018), order of 19 May 2023 (NGT via Indian Kanoon, 2023): Compensation 'on the scale of Rs. 2 crore per MLD for gap in respect of liquid waste'; 'worked out in the light of scientific studies and cost of remediation' https://indiankanoon.org/doc/5883219</t>
         </is>
       </c>
       <c r="N61" s="11" t="inlineStr">
         <is>
-          <t>How is the Rupees 42 per tree going to be spent (Isha Foundation (Cauvery Calling), 2019): Cauvery Calling: 'support farmers to plant 242 crore trees'; average cost Rs 42 per sapling https://isha.sadhguru.org/en/wisdom/article/rupees-42-per-tree-spent-cauvery-calling</t>
+          <t>NGT Central Zone order (CPCB environmental compensation method) (NGT, 2024): CPCB method assumes STP capital ₹1.75 cr/MLD, conveyance ₹5.55 cr/MLD and annual O&amp;M at 10% of combined capital https://www.greentribunal.gov.in/gen_pdf_test.php?filepath=L25ndF9kb2N1bWVudHMvbmd0L2Nhc2Vkb2MvanVkZ2VtZW50cy9CSE9QQUwvMjAyNC0wNC0wOC8xNzEyNTY5NzY1Njg4MjQ2NTE2NjYxM2JkYTU3MWVmYy5wZGY%3D</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>basin_loss</t>
+          <t>catchment_rs_kl</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
@@ -11669,21 +11903,21 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Share of the city's sewage that drains out of the Cauvery basin</t>
+          <t>Bengaluru's share of keeping the catchment forested</t>
         </is>
       </c>
       <c r="D62" s="11" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E62" s="11" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="F62" s="11" t="n">
-        <v>0.7</v>
+        <v>6</v>
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>₹/kL drawn</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
@@ -11693,54 +11927,59 @@
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Bengaluru drains through three valleys. The Hebbal and Koramangala–Challaghatta valleys flow east to the Dakshina Pinakini (South Pennar) and the Kolar tanks, outside the Cauvery basin. The Vrishabhavathi valley flows to the Arkavathy and back into the Cauvery. The Vrishabhavathi share of sewage is roughly a third to 40%, so about 60% of the draw is lost to the basin.</t>
+          <t>Natural forest in Kodagu and the Western Ghats keeps the river flowing in the dry months. Bengaluru pays nothing toward it. Its share of Cauvery Calling's costs comes to about ₹0.40/kL; Quito's water fund takes about 2% of utility revenue; New York spends about ₹7/kL at market exchange rates (about ₹1.5 at purchasing-power parity). ₹1 is a middle figure.</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr">
         <is>
-          <t>The valley split of sewage is approximate; no official figure was found. The polluted return flow through the Arkavathy is covered by the cost of treating sewage, not by this line.</t>
+          <t>A payment to keep the service, not compensation for damage.</t>
         </is>
       </c>
       <c r="K62" s="11" t="inlineStr">
         <is>
-          <t>Wastewater management in a metropolis: Bengaluru case study (S. Vishwanath, Biome Environmental Trust (CSE), 2022): Three valleys (K&amp;C, Hebbal, Vrishabhavathi); treated water conveyed to Kolar, Chikkaballapur and V-Valley tanks https://cdn.cseindia.org/attachments/0.64097500_1670989641_wastewater-management-in-a-metropolis-(bengaluru-case-study)-by-s-vishwanath,-biome-environmental-trust.pdf</t>
+          <t>Cauvery Calling (Isha Outreach, None): Programme to plant trees across the Cauvery basin, about ₹42 per tree https://www.ishaoutreach.org/en/cauvery-calling</t>
         </is>
       </c>
       <c r="L62" s="11" t="inlineStr">
         <is>
-          <t>How Bengaluru's domestic wastewater is helping parched Kolar (IndiaSpend, 2019): K-C Valley sends 440 MLD of treated sewage east to Kolar tanks https://www.indiaspend.com/how-bengalurus-domestic-wastewater-is-helping-parched-kolar</t>
+          <t>Isha says 13.4 crore trees planted under Cauvery Calling (The Week, 2026): 13.4 crore trees planted by 2026 https://www.theweek.in/news/india/2026/05/29/isha-foundation-says-13-4-crore-trees-planted-under-cauvery-calling-sets-1-2-crore-target-for-2026-27.html</t>
         </is>
       </c>
       <c r="M62" s="11" t="inlineStr">
         <is>
-          <t>Bengaluru urban water balance (WELL Labs, 2024): City water balance by valley, including outflows via Vrishabhavathi to the Arkavathy https://welllabs.org/wp-content/uploads/2024/03/Jan-2024_WELL-Labs-Bengaluru-Urban-Water-Balance-Report.pdf</t>
+          <t>Review of the New York City Watershed Protection Program (National Academies, 2020): Cost and results of New York's watershed programme https://www.nycwatershed.org/wp-content/uploads/2022/11/NAS-NYC-WPP-Review-2020.pdf</t>
+        </is>
+      </c>
+      <c r="N62" s="11" t="inlineStr">
+        <is>
+          <t>Payments for watershed services in Ecuador (FONAG) (CBD, None): Quito's water fund is financed by a share of the utility's revenue https://www.cbd.int/financial/pes/ecuador-peswater.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
         <is>
-          <t>raw_oc_rs_kl</t>
+          <t>eflow_rs_kl</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Scarcity and the river</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Value of Cauvery water to downstream farms</t>
+          <t>River flow for fish and wildlife in the dry months</t>
         </is>
       </c>
       <c r="D63" s="11" t="n">
         <v>4</v>
       </c>
       <c r="E63" s="11" t="n">
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="F63" s="11" t="n">
-        <v>11</v>
+        <v>7.3</v>
       </c>
       <c r="G63" s="11" t="inlineStr">
         <is>
@@ -11754,58 +11993,63 @@
       </c>
       <c r="I63" s="11" t="inlineStr">
         <is>
-          <t>Bengaluru's draw is a kL that Cauvery farmers downstream cannot use, at least for the share that leaves the basin. Paddy grown with that water in the delta is worth about ₹11 gross in a normal year; after costs, about ₹2–5. In drought years it is worth far more, so the range runs to ₹11.</t>
+          <t>When the river is held to a minimum flow, a kilolitre the city takes in the dry months has to come from somewhere else. The cheapest substitute we can price is recycled water at ₹12–15/kL. We assume that limit binds for about 30% of what the city draws (10–50%). 0.3 × ₹13.5 is about ₹4.</t>
         </is>
       </c>
       <c r="J63" s="11" t="inlineStr">
         <is>
-          <t>0.48 kg/m³ × ₹23.69/kg = ₹11.4/m³ gross (our calculation); a 20-40% net margin gives ₹2-5. No peer-reviewed Cauvery-delta value of water was found.</t>
+          <t>The least certain number on the page. No flow–ecology study exists for this reach. A cross-check using prices paid to buy water back for Australian and US rivers gives ₹0.75. When KRS has water, Karnataka can release more instead, at the cost of Mandya cane (₹1.5–6/kL). About 60% of the value is in the gorge above Sangama and is lost at the intake; the rest is in the sanctuary reach below Sangama, which returned water does reach.</t>
         </is>
       </c>
       <c r="K63" s="11" t="inlineStr">
         <is>
-          <t>Water productivity of paddy, Tamil Nadu (Madras Agricultural Journal, 2009): 0.48 kg rice per m³ of water https://masujournal.org/store_file/archive/96-7-12-353-355.pdf</t>
+          <t>Assessment of ecological status of Cauvery River (Wildlife Institute of India / NRCD, None): Cites the NGT direction to keep 25–30% of lean-season flow; recommends states fix and maintain e-flows https://v1.wii.gov.in/images/images/documents/ganga_project/NRCD_Cauvery_Report.pdf</t>
         </is>
       </c>
       <c r="L63" s="11" t="inlineStr">
         <is>
-          <t>Centre raises paddy MSP to ₹2,369/quintal for 2025-26 (Deccan Herald, 2025): Paddy MSP ₹2,369 per quintal https://www.deccanherald.com/business/centre-raises-paddy-msp-by-rs-69-to-rs-2369-per-quintal-for-2025-26-3560683</t>
+          <t>Rajya Sabha answer on Cauvery releases (Parliament of India, 2026): Stipulated monthly flows at Biligundlu: 2.5 TMC a month in Feb–May, about 27 m³/s https://sansad.in/getFile/annex/265/AU89_Nzt2sT.pdf?source=pqars</t>
         </is>
       </c>
       <c r="M63" s="11" t="inlineStr">
         <is>
-          <t>India Water Resource Report (ICRIER, 2019): Farm groundwater costs ₹2.1-2.8 per m³ in TN and Gujarat https://icrier.org/pdf/ICRIER_Water_Resource_Report_2019.pdf</t>
+          <t>Cost-benefit analysis of the K-C Valley treated-water scheme (preprint) (Research Square (IISc authors), 2023): Recycled water costs ₹12.43/kL at 5% and ₹14.61/kL at 8%; farm income gain about ₹80/kL gross https://www.researchsquare.com/article/rs-3401470/latest.pdf</t>
+        </is>
+      </c>
+      <c r="N63" s="11" t="inlineStr">
+        <is>
+          <t>Effects of water recovery on the southern Murray–Darling water market (Murray–Darling Basin Authority, 2025): Prices paid to buy water back for rivers (benefit-transfer check) https://www.mdba.gov.au/sites/default/files/publications/bcmp-effects-water-recovery-southern-mbb-water-market.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>lrmc_cr_mld</t>
+          <t>hydro_w_rs_kl</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>Scarcity and the river</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Cost of the next source (Stage VI: ₹6,939 cr / 500 MLD)</t>
+          <t>Hydropower lost at Shivanasamudram</t>
         </is>
       </c>
       <c r="D64" s="11" t="n">
-        <v>13.9</v>
+        <v>0.57</v>
       </c>
       <c r="E64" s="11" t="n">
-        <v>10.3</v>
+        <v>0.35</v>
       </c>
       <c r="F64" s="11" t="n">
-        <v>16</v>
+        <v>1.66</v>
       </c>
       <c r="G64" s="11" t="inlineStr">
         <is>
-          <t>₹ cr/MLD</t>
+          <t>₹/kL drawn</t>
         </is>
       </c>
       <c r="H64" s="11" t="inlineStr">
@@ -11815,737 +12059,718 @@
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>Cauvery Stage VI is budgeted at ₹6,939 crore for 500 MLD, about twice Stage V per MLD. It is used for the price signal in the top tariff block, not in the cost ladder.</t>
+          <t>Bengaluru draws at the Shiva Anicut, which also feeds the Shivanasamudram power channel (126.5 m head). Each kL not turbined loses about 0.3 units of power. The station is short of water for part of the year, so roughly 30–70% of the draw (about 37% in a normal year) is power lost, valued at ₹3.9–7.8 a unit.</t>
         </is>
       </c>
       <c r="J64" s="11" t="inlineStr">
         <is>
-          <t>NIE (Aug 2026) puts Stage VI at 675 MLD, which would cut the rate to ~₹10.3 cr/MLD. Mekedatu (₹16,745 cr revised DPR) is multi-purpose and is not used.</t>
+          <t>Zero if Karnataka releases extra water from KRS to cover the city; then the cost falls on Karnataka's farms instead.</t>
         </is>
       </c>
       <c r="K64" s="11" t="inlineStr">
         <is>
-          <t>Karnataka Budget 2026-27, para 304 (Govt of Karnataka, 2026): Cauvery Phase VI ₹6,939 cr with JICA for 6 TMC https://cm.karnataka.gov.in/uploads/media_to_upload1772784239.pdf</t>
+          <t>Report on east-flowing rivers of peninsular India (hydro potential) (Central Electricity Authority, 2023): Shivasamudram 42 MW at 126.49 m rated head; Mettur and barrage stations with heads and generation https://cea.nic.in/wp-content/uploads/2023/07/ReportonEastFlowingRiversPeninsulaIndia%28EFR%29.pdf</t>
         </is>
       </c>
       <c r="L64" s="11" t="inlineStr">
         <is>
-          <t>Bengaluru to draw more Cauvery water: Stage VI (Deccan Herald, 2025): ₹6,939 cr DPR for 500 MLD https://www.deccanherald.com/india/karnataka/bengaluru/bengaluru-to-draw-more-cauvery-water-cm-siddaramaiah-announces-sixth-phase-3235353</t>
+          <t>All station performance, April 2024 (Karnataka Power Corporation, 2024): Monthly generation at Shivasamudram, low in the dry months https://kpcl.karnataka.gov.in/storage/pdf-files/AllstationperformanceApril2024.pdf</t>
         </is>
       </c>
       <c r="M64" s="11" t="inlineStr">
         <is>
-          <t>BWSSB plans solar-powered upgrade for Cauvery Stage 6 (Bangalore Mirror, 2025): Cites a ₹5,177 cr DPR (KRS via Ramanagara bypass) https://bangaloremirror.indiatimes.com/bangalore/others/bwssb-plans-solar-powered-upgrade-for-cauvery-stage-6/articleshow/124278554.cms</t>
+          <t>Market monitoring annual report 2024-25 (CERC, 2025): Exchange power prices used to value lost generation https://www.cercind.gov.in/2025/market_monitoring/Annual-Report-2024-25.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
         <is>
-          <t>gw_share</t>
+          <t>hydro_n_rs_kl</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>Scarcity and the river</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Share of city demand met by groundwater</t>
+          <t>Hydropower lost at Mettur and the Tamil Nadu barrages</t>
         </is>
       </c>
       <c r="D65" s="11" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="E65" s="11" t="n">
         <v>0.4</v>
       </c>
-      <c r="E65" s="11" t="n">
-        <v>0.15</v>
-      </c>
       <c r="F65" s="11" t="n">
-        <v>0.52</v>
+        <v>1.62</v>
       </c>
       <c r="G65" s="11" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>₹/kL not returned</t>
         </is>
       </c>
       <c r="H65" s="11" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="I65" s="11" t="inlineStr">
         <is>
-          <t>Borewells and tankers fill the gap that Cauvery water leaves. WELL Labs' 2026 water balance puts groundwater at about 40% of demand; official figures are lower.</t>
+          <t>Water that never returns to the Cauvery would have run through Mettur, Lower Mettur and the barrage power houses: about 102 m of fall in all. Valued the same way.</t>
         </is>
       </c>
       <c r="J65" s="11" t="inlineStr"/>
       <c r="K65" s="11" t="inlineStr">
         <is>
-          <t>Why Bengaluru should reuse treated used water (WELL Labs, 2026): ~40% of demand met by groundwater https://welllabs.org/why-bengaluru-should-reuse-treated-used-water</t>
+          <t>Report on east-flowing rivers of peninsular India (hydro potential) (Central Electricity Authority, 2023): Shivasamudram 42 MW at 126.49 m rated head; Mettur and barrage stations with heads and generation https://cea.nic.in/wp-content/uploads/2023/07/ReportonEastFlowingRiversPeninsulaIndia%28EFR%29.pdf</t>
         </is>
       </c>
       <c r="L65" s="11" t="inlineStr">
         <is>
-          <t>Bengaluru Urban Water Balance Report (WELL Labs, 2024): Groundwater ~52% of supply (Jan 2024 version) https://welllabs.org/wp-content/uploads/2024/03/Jan-2024_WELL-Labs-Bengaluru-Urban-Water-Balance-Report.pdf</t>
+          <t>Statistical handbook: electricity (Tamil Nadu DES, 2025): Generation at Mettur and Cauvery barrage power houses https://des.tn.gov.in/sites/default/files/2025-07/10.%20ELECTRICITY.pdf</t>
         </is>
       </c>
       <c r="M65" s="11" t="inlineStr">
         <is>
-          <t>Bengaluru facing shortfall of 500 MLD: CM (New Indian Express, 2024): Need 2,600 MLD: 1,470 Cauvery + 650 borewells (~25%) https://www.newindianexpress.com/cities/bengaluru/2024/Mar/18/bengaluru-facing-shortfall-of-500-mld-water-karnataka-cm</t>
-        </is>
-      </c>
-      <c r="N65" s="11" t="inlineStr">
-        <is>
-          <t>Water supply to core city ramped up (chairman interview) (New Indian Express, 2026): ~400 MLD from groundwater against 2,600 MLD need (~15%) https://www.newindianexpress.com/cities/bengaluru/2026/May/18/water-supply-to-core-city-ramped-up-pipeline-network-for-suburbs-under-way-bwssb-chairman</t>
+          <t>Market monitoring annual report 2024-25 (CERC, 2025): Exchange power prices used to value lost generation https://www.cercind.gov.in/2025/market_monitoring/Annual-Report-2024-25.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>grid_ef</t>
+          <t>delta_rs_kl</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>Carbon</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Grid emission factor (CEA v22, FY26)</t>
+          <t>Delta and coast: seawater intrusion, mangroves</t>
         </is>
       </c>
       <c r="D66" s="11" t="n">
-        <v>0.675</v>
+        <v>0.3</v>
       </c>
       <c r="E66" s="11" t="n">
-        <v>0.512</v>
+        <v>0</v>
       </c>
       <c r="F66" s="11" t="n">
-        <v>0.727</v>
+        <v>1.5</v>
       </c>
       <c r="G66" s="11" t="inlineStr">
         <is>
-          <t>tCO₂/MWh</t>
+          <t>₹/kL not returned</t>
         </is>
       </c>
       <c r="H66" s="11" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>assumed</t>
         </is>
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>India's Central Electricity Authority puts average grid emissions at 0.675 tonnes of CO₂ per MWh for FY2025-26, the latest figure.</t>
-        </is>
-      </c>
-      <c r="J66" s="11" t="inlineStr"/>
+          <t>Less fresh water reaching the delta lets seawater into rivers and wells. Tamil Nadu is spending heavily on barrages to hold it back. Only a small share of that can be pinned on Bengaluru's draw, hence ₹0.3.</t>
+        </is>
+      </c>
+      <c r="J66" s="11" t="inlineStr">
+        <is>
+          <t>Overlaps with farm value; kept small to avoid counting the same harm twice.</t>
+        </is>
+      </c>
       <c r="K66" s="11" t="inlineStr">
         <is>
-          <t>CO₂ Baseline Database v22.0 (Central Electricity Authority, 2026): FY2025-26 weighted average 0.675 tCO₂/MWh https://cea.nic.in/api/cdm-report-version/view-pdf/en/82</t>
+          <t>Climate adaptation in Vennar subbasin (report and recommendation) (Asian Development Bank, None): Delta works against seawater intrusion and flooding https://www.adb.org/sites/default/files/project-documents//44429-013-rrp.pdf</t>
         </is>
       </c>
       <c r="L66" s="11" t="inlineStr">
         <is>
-          <t>CO₂ Baseline Database v21.0 (Central Electricity Authority, 2025): FY2024-25 weighted average 0.710; build margin 0.512 https://cea.nic.in/api/cdm-report-version/view-pdf/en/78</t>
+          <t>₹972 crore plan to protect three rivers from seawater intrusion (New Indian Express, 2026): Tamil Nadu plans ₹972 crore of barrages against seawater in delta rivers https://www.newindianexpress.com/states/tamil-nadu/2026/Aug/29/rs-972-crore-plan-to-protect-three-rivers-from-seawater-intrusion-tn-water-resources-minister-n-anand</t>
         </is>
       </c>
       <c r="M66" s="11" t="inlineStr">
         <is>
-          <t>CEA version 21 vs 22 grid factor revisions (Senseible, 2026): v22 FY26 0.675; excluding imports 0.678 https://senseible.earth/answers/cea-version-21-vs-22-grid-factor-revisions</t>
+          <t>How valuable are mangroves? Study on Pichavaram (The Hindu, 2026): Ecosystem value of the Pichavaram mangroves https://www.thehindu.com/news/national/karnataka/how-valuable-are-mangroves-study-on-pichavaram-ecosystem-pegs-it-at-248538-crore/article71419454.ece</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>scc_usd</t>
+          <t>gwrech_rs_kl</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>Carbon</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>Social cost of carbon</t>
+          <t>Groundwater recharge downstream</t>
         </is>
       </c>
       <c r="D67" s="11" t="n">
-        <v>255</v>
+        <v>0.12</v>
       </c>
       <c r="E67" s="11" t="n">
-        <v>40</v>
+        <v>0.03</v>
       </c>
       <c r="F67" s="11" t="n">
-        <v>425</v>
+        <v>0.4</v>
       </c>
       <c r="G67" s="11" t="inlineStr">
         <is>
-          <t>$/tCO₂</t>
+          <t>₹/kL not returned</t>
         </is>
       </c>
       <c r="H67" s="11" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>Carbon dioxide does damage worldwide, so it is valued at global damages: the US EPA's 2023 central estimate for emissions in 2025–26, about $210 a tonne in 2020 dollars, or about $255 in 2026 dollars. The low end, about $40, is India's own share of global damages on the same basis. The high end, about $425, is EPA's value at a 1.5% discount rate.</t>
+          <t>River flow and canal seepage refill wells downstream. Valued at the pumping energy farmers save.</t>
         </is>
       </c>
       <c r="J67" s="11" t="inlineStr">
         <is>
-          <t>The US withdrew these estimates from federal use in 2025; the science behind them has not changed. Ricke et al. (2018) give India's country-level cost as about $86, but that sits on a scale whose global median is $417, so it is not comparable with EPA's figure.</t>
+          <t>Mostly already inside farm returns.</t>
         </is>
       </c>
       <c r="K67" s="11" t="inlineStr">
         <is>
-          <t>Report on the Social Cost of Greenhouse Gases (US EPA, 2023): SC-CO₂ for 2020 emissions: $120 / $190 / $340 at 2.5% / 2.0% / 1.5% (2020$) https://www.epa.gov/system/files/documents/2023-12/epa_scghg_2023_report_final.pdf</t>
+          <t>Dynamic groundwater resources (CGWB, 2024): Recharge from canals and rivers in Cauvery districts https://cgwb.gov.in/cgwbpnm/public/uploads/documents/17357169591419696804file.pdf</t>
         </is>
       </c>
       <c r="L67" s="11" t="inlineStr">
         <is>
-          <t>Comprehensive evidence implies a higher social cost of CO₂ (Nature (Rennert et al.), 2022): Mean $185/tCO₂ (5-95%: $44-413) at 2% discount rate https://www.nature.com/articles/s41586-022-05224-9</t>
-        </is>
-      </c>
-      <c r="M67" s="11" t="inlineStr">
-        <is>
-          <t>Country-level social cost of carbon (Nature Climate Change (Ricke et al.), 2018): India's country-level SCC is the world's highest, ~$86/tCO₂ (median as reported) https://ideas.repec.org/a/nat/natcli/v8y2018i10d10.1038_s41558-018-0282-y.html</t>
-        </is>
-      </c>
-      <c r="N67" s="11" t="inlineStr">
-        <is>
-          <t>Social Cost of Greenhouse Gases: background and recent developments (Congressional Research Service, 2025): EO 14154 (20 Jan 2025) directed US agencies to stop using the SC-GHG estimates https://www.congress.gov/crs_external_products/IF/HTML/IF12916.html</t>
+          <t>Measuring the marginal value of water (Kolar) (Somanathan &amp; Ravindranath, EPW, 2006): Groundwater sales in Kolar at a mean ₹0.58/m³ (2006 prices) https://www.isid.ac.in/~som/papers/watervalueEPW.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>fx</t>
+          <t>kolar_rs_kl</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>Carbon</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Exchange rate (FBIL, 30 Oct 2026)</t>
+          <t>Value of treated water to Kolar and Chikkaballapur farmers</t>
         </is>
       </c>
       <c r="D68" s="11" t="n">
-        <v>95.25</v>
+        <v>15</v>
       </c>
       <c r="E68" s="11" t="n">
-        <v>94.40000000000001</v>
+        <v>5</v>
       </c>
       <c r="F68" s="11" t="n">
-        <v>96.8</v>
+        <v>30</v>
       </c>
       <c r="G68" s="11" t="inlineStr">
         <is>
-          <t>₹/$</t>
+          <t>₹/kL</t>
         </is>
       </c>
       <c r="H68" s="11" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>Used only to turn the dollar carbon price into rupees. The official FBIL reference rate on 30 October 2026 was ₹95.25 per dollar.</t>
-        </is>
-      </c>
-      <c r="J68" s="11" t="inlineStr"/>
+          <t>An IISc team's study of the K-C Valley scheme finds about ₹80 of extra farm income per kL gross. After costs and attribution, about ₹20 on average. The next kL, into tanks already fuller, is worth less, so ₹15 is used. Charged only if the city pipes this water back to the Cauvery instead.</t>
+        </is>
+      </c>
+      <c r="J68" s="11" t="inlineStr">
+        <is>
+          <t>Based on one preprint that has not been peer reviewed.</t>
+        </is>
+      </c>
       <c r="K68" s="11" t="inlineStr">
         <is>
-          <t>FBIL reference rate (RBI homepage) (Reserve Bank of India / FBIL, 2026): ₹95.2492 per USD, 30 Oct 2026 https://www.rbi.org.in/</t>
+          <t>Cost-benefit analysis of the K-C Valley treated-water scheme (preprint) (Research Square (IISc authors), 2023): Recycled water costs ₹12.43/kL at 5% and ₹14.61/kL at 8%; farm income gain about ₹80/kL gross https://www.researchsquare.com/article/rs-3401470/latest.pdf</t>
         </is>
       </c>
       <c r="L68" s="11" t="inlineStr">
         <is>
-          <t>USD to INR history 2026 (Pound Sterling Live, 2026): October 2026 range ~₹94.4-96.8 https://www.poundsterlinglive.com/history/USD-INR-2026</t>
+          <t>Kolar water table rises 50–100 ft under K-C Valley project, says IISc (The Hindu, 2026): Water tables up 50–100 ft; no harm found to soil, crops or livestock https://www.thehindu.com/news/cities/bangalore/kolar-water-table-rises-to-50-100-ft-under-kc-valley-project-says-iisc/article70776124.ece</t>
+        </is>
+      </c>
+      <c r="M68" s="11" t="inlineStr">
+        <is>
+          <t>Drought-hit farmers in Kolar grow crops with treated wastewater (The News Minute, 2019): Farmers depend on K-C Valley water https://www.thenewsminute.com/karnataka/drought-hit-farmers-kolar-grow-crops-treated-wastewater-there-risk-101213</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
         <is>
-          <t>residual_rs_kl</t>
+          <t>basin_loss</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>Climate and residual harm</t>
+          <t>The river, the lakes and the catchment</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Residual harm after treating sewage to NGT norms</t>
+          <t>Share of the city's sewage that drains out of the Cauvery basin</t>
         </is>
       </c>
       <c r="D69" s="11" t="n">
-        <v>8</v>
+        <v>0.6</v>
       </c>
       <c r="E69" s="11" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="F69" s="11" t="n">
-        <v>12</v>
+        <v>0.7</v>
       </c>
       <c r="G69" s="11" t="inlineStr">
         <is>
-          <t>₹/kL sewage</t>
+          <t>share</t>
         </is>
       </c>
       <c r="H69" s="11" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>assumed</t>
         </is>
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>Even a plant meeting the strictest Indian norms still emits nitrous oxide and methane and releases some nitrogen and phosphorus. Priced with standard damage values, this comes to a few rupees per kilolitre of sewage.</t>
+          <t>Bengaluru drains through three valleys. The Hebbal and Koramangala–Challaghatta valleys flow east to the Dakshina Pinakini (South Pennar) and the Kolar tanks, outside the Cauvery basin. The Vrishabhavathi valley flows to the Arkavathy and back into the Cauvery. The Vrishabhavathi share of sewage is roughly a third to 40%, so about 60% of the draw is lost to the basin.</t>
         </is>
       </c>
       <c r="J69" s="11" t="inlineStr">
         <is>
-          <t>Worked with IPCC 2019 default factors and EPA damage values, the residual comes to about ₹8.7 per kL of sewage. The central value is set at 8, with a range of 3–12, because the nitrogen and sludge terms are uncertain.</t>
+          <t>The valley split of sewage is approximate; no official figure was found. The polluted return flow through the Arkavathy is covered by the cost of treating sewage, not by this line.</t>
         </is>
       </c>
       <c r="K69" s="11" t="inlineStr">
         <is>
-          <t>2019 Refinement, Vol 5 Ch 6: Wastewater Treatment and Discharge (IPCC, 2019): Table 6A.4: default N2O EF for domestic WWTPs 0.016 kg N2O-N/kg N (SD 0.012; range 0.00016-0.045) https://www.ipcc-nggip.iges.or.jp/public/2019rf/pdf/5_Volume5/19R_V5_6_Ch06_Wastewater.pdf</t>
+          <t>Wastewater management in a metropolis: Bengaluru case study (S. Vishwanath, Biome Environmental Trust (CSE), 2022): Three valleys (K&amp;C, Hebbal, Vrishabhavathi); treated water conveyed to Kolar, Chikkaballapur and V-Valley tanks https://cdn.cseindia.org/attachments/0.64097500_1670989641_wastewater-management-in-a-metropolis-(bengaluru-case-study)-by-s-vishwanath,-biome-environmental-trust.pdf</t>
         </is>
       </c>
       <c r="L69" s="11" t="inlineStr">
         <is>
-          <t>Comment: Updated estimates of the social cost of greenhouse gases (Regulations.gov (EPA docket), 2023): Central EPA estimates for 2020 emissions: $190/t CO2, $1,600/t CH4, $54,000/t N2O https://downloads.regulations.gov/EPA-HQ-OAR-2023-0072-0618/attachment_1.pdf</t>
+          <t>How Bengaluru's domestic wastewater is helping parched Kolar (IndiaSpend, 2019): K-C Valley sends 440 MLD of treated sewage east to Kolar tanks https://www.indiaspend.com/how-bengalurus-domestic-wastewater-is-helping-parched-kolar</t>
         </is>
       </c>
       <c r="M69" s="11" t="inlineStr">
         <is>
-          <t>Impact assessment, proposal to recast the Urban Wastewater Treatment Directive (European Commission, 2022): Shadow prices used for benefits: €20 per kg N and €30 per kg P removed; GHG €100/t CO2e https://environment.ec.europa.eu/system/files/2022-10/Impact%20assessment%20accompanying%20the%20proposal.pdf</t>
-        </is>
-      </c>
-      <c r="N69" s="11" t="inlineStr">
-        <is>
-          <t>Compendium of recycle and reuse of wastewater (NITI for States, 2022): Bengaluru STP inflows: total nitrogen 39-40 mg/L (e.g. Cubbon Park STP 40 mg/L in, &lt;10 out) https://www.nitiforstates.gov.in/public-assets/Policy/policy_files/RNC518E000039.pdf</t>
+          <t>Bengaluru urban water balance (WELL Labs, 2024): City water balance by valley, including outflows via Vrishabhavathi to the Arkavathy https://welllabs.org/wp-content/uploads/2024/03/Jan-2024_WELL-Labs-Bengaluru-Urban-Water-Balance-Report.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>re_share</t>
+          <t>lrmc_cr_mld</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>Climate and residual harm</t>
+          <t>Scarcity and the river</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Share of BWSSB power bought from renewables</t>
+          <t>Cost of the next source (Stage VI: ₹6,939 cr / 500 MLD)</t>
         </is>
       </c>
       <c r="D70" s="11" t="n">
-        <v>0</v>
+        <v>13.9</v>
       </c>
       <c r="E70" s="11" t="n">
-        <v>0</v>
+        <v>10.3</v>
       </c>
       <c r="F70" s="11" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G70" s="11" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>₹ cr/MLD</t>
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>BWSSB buys grid power today. It plans to run Stage VI pumping partly on solar, which would cut that scheme's power bill by about 30%; the slider shows what more green power would do to the carbon cost.</t>
+          <t>Cauvery Stage VI is budgeted at ₹6,939 crore for 500 MLD, about twice Stage V per MLD. It is used for the price signal in the top tariff block, not in the cost ladder.</t>
         </is>
       </c>
       <c r="J70" s="11" t="inlineStr">
         <is>
-          <t>Value 0 reflects today's grid purchases (the grid emission factor already counts the grid's own renewables). Stage VI estimate: ₹19.13 → ₹13.35 cr/month with solar. Green power from BESCOM costs 50 paise/unit extra; KERC's MW-scale solar benchmark is ₹3.04/unit vs the ₹6.25/kWh HT-1 energy charge.</t>
+          <t>NIE (Aug 2026) puts Stage VI at 675 MLD, which would cut the rate to ~₹10.3 cr/MLD. Mekedatu (₹16,745 cr revised DPR) is multi-purpose and is not used.</t>
         </is>
       </c>
       <c r="K70" s="11" t="inlineStr">
         <is>
-          <t>BWSSB plans solar-powered upgrade for Cauvery Stage 6 (Bangalore Mirror, 2025): Stages 1-5 power ~₹86.07 cr/month; Stage 6 (500 MLD) ₹19.13 cr/month on grid, ₹13.35 cr with solar; '₹5,177 crore DPR' https://bangaloremirror.indiatimes.com/bangalore/others/bwssb-plans-solar-powered-upgrade-for-cauvery-stage-6/articleshow/124278554.cms</t>
+          <t>Karnataka Budget 2026-27, para 304 (Govt of Karnataka, 2026): Cauvery Phase VI ₹6,939 cr with JICA for 6 TMC https://cm.karnataka.gov.in/uploads/media_to_upload1772784239.pdf</t>
         </is>
       </c>
       <c r="L70" s="11" t="inlineStr">
         <is>
-          <t>KERC Tariff Order 2025 (BESCOM) (KERC, 2025): Green tariff of 50 paise per unit over the normal tariff for HT consumers opting for green power https://kerc.karnataka.gov.in/uploads/96731743148968.pdf</t>
+          <t>Bengaluru to draw more Cauvery water: Stage VI (Deccan Herald, 2025): ₹6,939 cr DPR for 500 MLD https://www.deccanherald.com/india/karnataka/bengaluru/bengaluru-to-draw-more-cauvery-water-cm-siddaramaiah-announces-sixth-phase-3235353</t>
         </is>
       </c>
       <c r="M70" s="11" t="inlineStr">
         <is>
-          <t>KERC generic tariff for solar projects (1 Jul 2025 - 30 Jun 2026) (KERC, 2025): MW-scale solar benchmark tariff ₹3.04/unit; solar with battery storage ₹5.66/unit https://kerc.karnataka.gov.in/uploads/media_to_upload1752057190.pdf</t>
+          <t>BWSSB plans solar-powered upgrade for Cauvery Stage 6 (Bangalore Mirror, 2025): Cites a ₹5,177 cr DPR (KRS via Ramanagara bypass) https://bangaloremirror.indiatimes.com/bangalore/others/bwssb-plans-solar-powered-upgrade-for-cauvery-stage-6/articleshow/124278554.cms</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="11" t="inlineStr">
         <is>
-          <t>fixed_charge</t>
+          <t>gw_share</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Scarcity and the river</t>
         </is>
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Fixed charge per connection</t>
+          <t>Share of city demand met by groundwater</t>
         </is>
       </c>
       <c r="D71" s="11" t="n">
-        <v>100</v>
+        <v>0.4</v>
       </c>
       <c r="E71" s="11" t="n">
-        <v>50</v>
+        <v>0.15</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>150</v>
+        <v>0.52</v>
       </c>
       <c r="G71" s="11" t="inlineStr">
         <is>
-          <t>₹/connection/month</t>
+          <t>share</t>
         </is>
       </c>
       <c r="H71" s="11" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>Much of a water system's cost is fixed, so many utilities charge a monthly fee per connection on top of the per-kilolitre rate. ₹100 is close to what Delhi charges and what BWSSB already collects as meter charges.</t>
-        </is>
-      </c>
-      <c r="J71" s="11" t="inlineStr">
-        <is>
-          <t>BWSSB's meter charge today runs ₹30-150/month by slab; Delhi's service charge is ₹146.41 up to 20 kL. A high fixed charge falls hardest on small users, which is why it is kept modest.</t>
-        </is>
-      </c>
+          <t>Borewells and tankers fill the gap that Cauvery water leaves. WELL Labs' 2026 water balance puts groundwater at about 40% of demand; official figures are lower.</t>
+        </is>
+      </c>
+      <c r="J71" s="11" t="inlineStr"/>
       <c r="K71" s="11" t="inlineStr">
         <is>
-          <t>Revised Water Tariff Ready Reckoner 2025 (BWSSB, 2025): Domestic: 0-8 kL ₹8.5 (min ₹68), 8-25 ₹14, 25-50 ₹34, &gt;50 ₹55; sanitary ₹14 flat up to 8 kL; meter charge ₹30/50/75/150; bulk ₹99/kL; 3% auto increase each 1 April https://bwssb.karnataka.gov.in/storage/pdf-files/WaterTariff-2025.pdf</t>
+          <t>Why Bengaluru should reuse treated used water (WELL Labs, 2026): ~40% of demand met by groundwater https://welllabs.org/why-bengaluru-should-reuse-treated-used-water</t>
         </is>
       </c>
       <c r="L71" s="11" t="inlineStr">
         <is>
-          <t>Water tariff (Delhi Jal Board, 2026): Domestic service charge ₹146.41/month up to 20 kL (₹219.62 for 20-30 kL, ₹292.82 above 30); free up to 20 kL with a functional meter; above 20 kL full consumption billed https://delhijalboard.delhi.gov.in/jalboard/about-us</t>
+          <t>Bengaluru Urban Water Balance Report (WELL Labs, 2024): Groundwater ~52% of supply (Jan 2024 version) https://welllabs.org/wp-content/uploads/2024/03/Jan-2024_WELL-Labs-Bengaluru-Urban-Water-Balance-Report.pdf</t>
         </is>
       </c>
       <c r="M71" s="11" t="inlineStr">
         <is>
-          <t>Pricing Water Resources and Water and Sanitation Services (OECD, 2010): Countries are moving to 'two-part tariffs combining fixed charges and variable fees'; large share of fixed costs 'would call for their recovery through fixed charges' https://www.oecd.org/content/dam/oecd/en/publications/reports/2010/03/pricing-water-resources-and-water-and-sanitation-services_g1ghc680/9789264083608-en.pdf</t>
+          <t>Bengaluru facing shortfall of 500 MLD: CM (New Indian Express, 2024): Need 2,600 MLD: 1,470 Cauvery + 650 borewells (~25%) https://www.newindianexpress.com/cities/bengaluru/2024/Mar/18/bengaluru-facing-shortfall-of-500-mld-water-karnataka-cm</t>
         </is>
       </c>
       <c r="N71" s="11" t="inlineStr">
         <is>
-          <t>Addressing the social consequences of tariffs for water supply and sanitation (OECD, 2020): Financial sustainability 'is likely to be strengthened if the tariff also includes a recurrent fixed charge', but fixed charges may raise social issues https://one.oecd.org/document/ENV/WKP(2020)13/En/pdf</t>
+          <t>Water supply to core city ramped up (chairman interview) (New Indian Express, 2026): ~400 MLD from groundwater against 2,600 MLD need (~15%) https://www.newindianexpress.com/cities/bengaluru/2026/May/18/water-supply-to-core-city-ramped-up-pipeline-network-for-suburbs-under-way-bwssb-chairman</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>b1_top</t>
+          <t>grid_ef</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Carbon</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Lifeline block: upper limit</t>
+          <t>Grid emission factor (CEA v22, FY26)</t>
         </is>
       </c>
       <c r="D72" s="11" t="n">
-        <v>10</v>
+        <v>0.675</v>
       </c>
       <c r="E72" s="11" t="n">
-        <v>8</v>
+        <v>0.512</v>
       </c>
       <c r="F72" s="11" t="n">
-        <v>15</v>
+        <v>0.727</v>
       </c>
       <c r="G72" s="11" t="inlineStr">
         <is>
-          <t>kL/month</t>
+          <t>tCO₂/MWh</t>
         </is>
       </c>
       <c r="H72" s="11" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>The first block should cover essential use at a low price. 10 kL a month is about 83 litres per person per day for a family of four: above WHO's 50-litre basic level, below the 135-litre planning norm.</t>
-        </is>
-      </c>
-      <c r="J72" s="11" t="inlineStr">
-        <is>
-          <t>4 × 50 L × 30 = 6 kL (WHO intermediate access); 4 × 100 L × 30 = 12 kL (top of OHCHR's 50-100 L); 4 × 135 L × 30 = 16.2 kL (CPHEEO). BWSSB's first slab is 8 kL; Delhi and Hyderabad give 20 kL free.</t>
-        </is>
-      </c>
+          <t>India's Central Electricity Authority puts average grid emissions at 0.675 tonnes of CO₂ per MWh for FY2025-26, the latest figure.</t>
+        </is>
+      </c>
+      <c r="J72" s="11" t="inlineStr"/>
       <c r="K72" s="11" t="inlineStr">
         <is>
-          <t>Domestic water quantity, service level and health (2nd ed.) (WHO, 2020): Intermediate access: average quantity about 50 L/person/day; optimal access (multiple taps) 100+ L https://www.who.int/publications/i/item/9789240015241</t>
+          <t>CO₂ Baseline Database v22.0 (Central Electricity Authority, 2026): FY2025-26 weighted average 0.675 tCO₂/MWh https://cea.nic.in/api/cdm-report-version/view-pdf/en/82</t>
         </is>
       </c>
       <c r="L72" s="11" t="inlineStr">
         <is>
-          <t>FAQ on the human right to water and sanitation (OHCHR, 2012): 20 L/person/day is a minimum; 'States should aim for at least 50 to 100 litres per person per day' https://www.ohchr.org/sites/default/files/Documents/Issues/Water/FAQWater_en.pdf</t>
+          <t>CO₂ Baseline Database v21.0 (Central Electricity Authority, 2025): FY2024-25 weighted average 0.710; build margin 0.512 https://cea.nic.in/api/cdm-report-version/view-pdf/en/78</t>
         </is>
       </c>
       <c r="M72" s="11" t="inlineStr">
         <is>
-          <t>Handbook on Service Level Benchmarking (MoUD (now MoHUA), 2010): Per capita supply of water: benchmark 135 lpcd https://mohua.gov.in/static/uploads/2025/10/627238a27786db8ce624ea6c3db6ae24.pdf</t>
-        </is>
-      </c>
-      <c r="N72" s="11" t="inlineStr">
-        <is>
-          <t>Revised Water Tariff Ready Reckoner 2025 (BWSSB, 2025): Domestic: 0-8 kL ₹8.5 (min ₹68), 8-25 ₹14, 25-50 ₹34, &gt;50 ₹55; sanitary ₹14 flat up to 8 kL; meter charge ₹30/50/75/150; bulk ₹99/kL; 3% auto increase each 1 April https://bwssb.karnataka.gov.in/storage/pdf-files/WaterTariff-2025.pdf</t>
+          <t>CEA version 21 vs 22 grid factor revisions (Senseible, 2026): v22 FY26 0.675; excluding imports 0.678 https://senseible.earth/answers/cea-version-21-vs-22-grid-factor-revisions</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="11" t="inlineStr">
         <is>
-          <t>b1_rate</t>
+          <t>scc_usd</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Carbon</t>
         </is>
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Lifeline block: rate (all-in)</t>
+          <t>Social cost of carbon</t>
         </is>
       </c>
       <c r="D73" s="11" t="n">
-        <v>15</v>
+        <v>255</v>
       </c>
       <c r="E73" s="11" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="F73" s="11" t="n">
-        <v>25</v>
+        <v>425</v>
       </c>
       <c r="G73" s="11" t="inlineStr">
         <is>
-          <t>₹/kL</t>
+          <t>$/tCO₂</t>
         </is>
       </c>
       <c r="H73" s="11" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>Today a household using 8 kL pays about ₹14.3 per kL all-in (water, sanitary and meter charges). Keeping the lifeline near that level protects the poorest from any increase.</t>
+          <t>Carbon dioxide does damage worldwide, so it is valued at global damages: the US EPA's 2023 central estimate for emissions in 2025–26, about $210 a tonne in 2020 dollars, or about $255 in 2026 dollars. The low end, about $40, is India's own share of global damages on the same basis. The high end, about $425, is EPA's value at a 1.5% discount rate.</t>
         </is>
       </c>
       <c r="J73" s="11" t="inlineStr">
         <is>
-          <t>FY27 bill at 8 kL: minimum ₹68 × 1.03 + sanitary ₹14 × 1.03 + meter ₹30 = ₹114.5 ÷ 8 = ₹14.3/kL. Chennai charges ₹8/kL up to 10 kL; Hyderabad ~₹10/kL with 20 kL free.</t>
+          <t>The US withdrew these estimates from federal use in 2025; the science behind them has not changed. Ricke et al. (2018) give India's country-level cost as about $86, but that sits on a scale whose global median is $417, so it is not comparable with EPA's figure.</t>
         </is>
       </c>
       <c r="K73" s="11" t="inlineStr">
         <is>
-          <t>Revised Water Tariff Ready Reckoner 2025 (BWSSB, 2025): Domestic: 0-8 kL ₹8.5 (min ₹68), 8-25 ₹14, 25-50 ₹34, &gt;50 ₹55; sanitary ₹14 flat up to 8 kL; meter charge ₹30/50/75/150; bulk ₹99/kL; 3% auto increase each 1 April https://bwssb.karnataka.gov.in/storage/pdf-files/WaterTariff-2025.pdf</t>
+          <t>Report on the Social Cost of Greenhouse Gases (US EPA, 2023): SC-CO₂ for 2020 emissions: $120 / $190 / $340 at 2.5% / 2.0% / 1.5% (2020$) https://www.epa.gov/system/files/documents/2023-12/epa_scghg_2023_report_final.pdf</t>
         </is>
       </c>
       <c r="L73" s="11" t="inlineStr">
         <is>
-          <t>Water and sewerage tariff (CMWSSB (Chennai), 2026): Domestic: up to 10 kL ₹8/kL, 11-15 ₹20, 16-25 ₹32, above 25 ₹51; minimum ₹111/month incl. sewer https://cmwssb.tn.gov.in/tariff</t>
+          <t>Comprehensive evidence implies a higher social cost of CO₂ (Nature (Rennert et al.), 2022): Mean $185/tCO₂ (5-95%: $44-413) at 2% discount rate https://www.nature.com/articles/s41586-022-05224-9</t>
         </is>
       </c>
       <c r="M73" s="11" t="inlineStr">
         <is>
-          <t>Water bills set to rise 5% every year as HMWSSB seeks to plug revenue gap (Times of India, 2026): Tariff about ₹10/kL; 20 kL free for about 5 lakh households; 5% annual hike https://timesofindia.indiatimes.com/city/hyderabad/water-bills-set-to-rise-5-every-yr-as-hmwssb-seeks-to-plug-revenue-gap/articleshow/134291436.cms</t>
+          <t>Country-level social cost of carbon (Nature Climate Change (Ricke et al.), 2018): India's country-level SCC is the world's highest, ~$86/tCO₂ (median as reported) https://ideas.repec.org/a/nat/natcli/v8y2018i10d10.1038_s41558-018-0282-y.html</t>
+        </is>
+      </c>
+      <c r="N73" s="11" t="inlineStr">
+        <is>
+          <t>Social Cost of Greenhouse Gases: background and recent developments (Congressional Research Service, 2025): EO 14154 (20 Jan 2025) directed US agencies to stop using the SC-GHG estimates https://www.congress.gov/crs_external_products/IF/HTML/IF12916.html</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>b2_top</t>
+          <t>fx</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Carbon</t>
         </is>
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Second block: upper limit</t>
+          <t>Exchange rate (FBIL, 30 Oct 2026)</t>
         </is>
       </c>
       <c r="D74" s="11" t="n">
-        <v>20</v>
+        <v>95.25</v>
       </c>
       <c r="E74" s="11" t="n">
-        <v>15</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="F74" s="11" t="n">
-        <v>30</v>
+        <v>96.8</v>
       </c>
       <c r="G74" s="11" t="inlineStr">
         <is>
-          <t>kL/month</t>
+          <t>₹/$</t>
         </is>
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>The second block covers ordinary family use up to the planning norm. A family of four at 135-150 litres a day uses 16-18 kL a month.</t>
-        </is>
-      </c>
-      <c r="J74" s="11" t="inlineStr">
-        <is>
-          <t>4 × 135 × 30 = 16.2 kL; 4 × 150 × 30 = 18 kL. Delhi's tariff steps at 20 and 30 kL.</t>
-        </is>
-      </c>
+          <t>Used only to turn the dollar carbon price into rupees. The official FBIL reference rate on 30 October 2026 was ₹95.25 per dollar.</t>
+        </is>
+      </c>
+      <c r="J74" s="11" t="inlineStr"/>
       <c r="K74" s="11" t="inlineStr">
         <is>
-          <t>Handbook on Service Level Benchmarking (MoUD (now MoHUA), 2010): Per capita supply of water: benchmark 135 lpcd https://mohua.gov.in/static/uploads/2025/10/627238a27786db8ce624ea6c3db6ae24.pdf</t>
+          <t>FBIL reference rate (RBI homepage) (Reserve Bank of India / FBIL, 2026): ₹95.2492 per USD, 30 Oct 2026 https://www.rbi.org.in/</t>
         </is>
       </c>
       <c r="L74" s="11" t="inlineStr">
         <is>
-          <t>CPHEEO Manual on Water Supply and Treatment (copy) (CPHEEO (Scribd copy), 1999): 135 lpcd for cities with sewerage; 150 lpcd for metropolitan and mega cities https://www.scribd.com/document/813009957/CPHEEO-Manual-on-Water-Supply</t>
-        </is>
-      </c>
-      <c r="M74" s="11" t="inlineStr">
-        <is>
-          <t>Water tariff (Delhi Jal Board, 2026): Domestic service charge ₹146.41/month up to 20 kL (₹219.62 for 20-30 kL, ₹292.82 above 30); free up to 20 kL with a functional meter; above 20 kL full consumption billed https://delhijalboard.delhi.gov.in/jalboard/about-us</t>
+          <t>USD to INR history 2026 (Pound Sterling Live, 2026): October 2026 range ~₹94.4-96.8 https://www.poundsterlinglive.com/history/USD-INR-2026</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="11" t="inlineStr">
         <is>
-          <t>b2_rate</t>
+          <t>residual_rs_kl</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Climate and residual harm</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Second block: rate</t>
+          <t>Residual harm after treating sewage to NGT norms</t>
         </is>
       </c>
       <c r="D75" s="11" t="n">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="E75" s="11" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="F75" s="11" t="n">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="G75" s="11" t="inlineStr">
         <is>
-          <t>₹/kL</t>
+          <t>₹/kL sewage</t>
         </is>
       </c>
       <c r="H75" s="11" t="inlineStr">
         <is>
-          <t>policy</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
-          <t>Normal household use should at least pay what it costs BWSSB to run the system today. BWSSB itself says it spends about ₹54 per kL; the model's cash cost per kL billed is about ₹62.</t>
+          <t>Even a plant meeting the strictest Indian norms still emits nitrous oxide and methane and releases some nitrogen and phosphorus. Priced with standard damage values, this comes to a few rupees per kilolitre of sewage.</t>
         </is>
       </c>
       <c r="J75" s="11" t="inlineStr">
         <is>
-          <t>Comparators: Chennai charges ₹51/kL above 25 kL; Delhi ₹26.36/kL (20-30 kL) plus 60% sewer = ₹42/kL plus service charge. ₹60 is roughly 4× today's ₹14/kL second slab.</t>
+          <t>Worked with IPCC 2019 default factors and EPA damage values, the residual comes to about ₹8.7 per kL of sewage. The central value is set at 8, with a range of 3–12, because the nitrogen and sludge terms are uncertain.</t>
         </is>
       </c>
       <c r="K75" s="11" t="inlineStr">
         <is>
-          <t>Water supply to core city ramped up (chairman interview) (New Indian Express, 2026): 'BWSSB spends around ₹54 per 1,000 litres to draw, treat and supply Cauvery water'; households pay ₹20-30/kL on average https://www.newindianexpress.com/cities/bengaluru/2026/May/18/water-supply-to-core-city-ramped-up-pipeline-network-for-suburbs-under-way-bwssb-chairman</t>
+          <t>2019 Refinement, Vol 5 Ch 6: Wastewater Treatment and Discharge (IPCC, 2019): Table 6A.4: default N2O EF for domestic WWTPs 0.016 kg N2O-N/kg N (SD 0.012; range 0.00016-0.045) https://www.ipcc-nggip.iges.or.jp/public/2019rf/pdf/5_Volume5/19R_V5_6_Ch06_Wastewater.pdf</t>
         </is>
       </c>
       <c r="L75" s="11" t="inlineStr">
         <is>
-          <t>Water and sewerage tariff (CMWSSB (Chennai), 2026): Domestic: up to 10 kL ₹8/kL, 11-15 ₹20, 16-25 ₹32, above 25 ₹51; minimum ₹111/month incl. sewer https://cmwssb.tn.gov.in/tariff</t>
+          <t>Comment: Updated estimates of the social cost of greenhouse gases (Regulations.gov (EPA docket), 2023): Central EPA estimates for 2020 emissions: $190/t CO2, $1,600/t CH4, $54,000/t N2O https://downloads.regulations.gov/EPA-HQ-OAR-2023-0072-0618/attachment_1.pdf</t>
         </is>
       </c>
       <c r="M75" s="11" t="inlineStr">
         <is>
-          <t>Economic Survey of Delhi 2023-24, Ch. 13 (Govt of NCT Delhi, 2024): Domestic tariff w.e.f. 01.02.2018: up to 20 kL ₹5.27/kL, 20-30 ₹26.36, &gt;30 ₹43.93 plus 60% sewer charge; non-domestic &gt;100 kL ₹175.69/kL https://delhiplanning.delhi.gov.in/sites/default/files/Planning/chapter_13.pdf</t>
+          <t>Impact assessment, proposal to recast the Urban Wastewater Treatment Directive (European Commission, 2022): Shadow prices used for benefits: €20 per kg N and €30 per kg P removed; GHG €100/t CO2e https://environment.ec.europa.eu/system/files/2022-10/Impact%20assessment%20accompanying%20the%20proposal.pdf</t>
+        </is>
+      </c>
+      <c r="N75" s="11" t="inlineStr">
+        <is>
+          <t>Compendium of recycle and reuse of wastewater (NITI for States, 2022): Bengaluru STP inflows: total nitrogen 39-40 mg/L (e.g. Cubbon Park STP 40 mg/L in, &lt;10 out) https://www.nitiforstates.gov.in/public-assets/Policy/policy_files/RNC518E000039.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>b3_top</t>
+          <t>re_share</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>A tariff that would work</t>
+          <t>Climate and residual harm</t>
         </is>
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Third block: upper limit</t>
+          <t>Share of BWSSB power bought from renewables</t>
         </is>
       </c>
       <c r="D76" s="11" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E76" s="11" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F76" s="11" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="G76" s="11" t="inlineStr">
         <is>
-          <t>kL/month</t>
+          <t>share</t>
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr">
@@ -12555,34 +12780,34 @@
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>Above about 40 kL a month a household is watering gardens or filling tanks, which is discretionary use. BWSSB's own third slab runs 25-50 kL.</t>
+          <t>BWSSB buys grid power today. It plans to run Stage VI pumping partly on solar, which would cut that scheme's power bill by about 30%; the slider shows what more green power would do to the carbon cost.</t>
         </is>
       </c>
       <c r="J76" s="11" t="inlineStr">
         <is>
-          <t>40 kL is more than twice the 18 kL a family of four needs at 150 lpcd. Delhi's top slab starts at 30 kL.</t>
+          <t>Value 0 reflects today's grid purchases (the grid emission factor already counts the grid's own renewables). Stage VI estimate: ₹19.13 → ₹13.35 cr/month with solar. Green power from BESCOM costs 50 paise/unit extra; KERC's MW-scale solar benchmark is ₹3.04/unit vs the ₹6.25/kWh HT-1 energy charge.</t>
         </is>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
-          <t>Revised Water Tariff Ready Reckoner 2025 (BWSSB, 2025): Domestic: 0-8 kL ₹8.5 (min ₹68), 8-25 ₹14, 25-50 ₹34, &gt;50 ₹55; sanitary ₹14 flat up to 8 kL; meter charge ₹30/50/75/150; bulk ₹99/kL; 3% auto increase each 1 April https://bwssb.karnataka.gov.in/storage/pdf-files/WaterTariff-2025.pdf</t>
+          <t>BWSSB plans solar-powered upgrade for Cauvery Stage 6 (Bangalore Mirror, 2025): Stages 1-5 power ~₹86.07 cr/month; Stage 6 (500 MLD) ₹19.13 cr/month on grid, ₹13.35 cr with solar; '₹5,177 crore DPR' https://bangaloremirror.indiatimes.com/bangalore/others/bwssb-plans-solar-powered-upgrade-for-cauvery-stage-6/articleshow/124278554.cms</t>
         </is>
       </c>
       <c r="L76" s="11" t="inlineStr">
         <is>
-          <t>CPHEEO Manual on Water Supply and Treatment (copy) (CPHEEO (Scribd copy), 1999): 135 lpcd for cities with sewerage; 150 lpcd for metropolitan and mega cities https://www.scribd.com/document/813009957/CPHEEO-Manual-on-Water-Supply</t>
+          <t>KERC Tariff Order 2025 (BESCOM) (KERC, 2025): Green tariff of 50 paise per unit over the normal tariff for HT consumers opting for green power https://kerc.karnataka.gov.in/uploads/96731743148968.pdf</t>
         </is>
       </c>
       <c r="M76" s="11" t="inlineStr">
         <is>
-          <t>Economic Survey of Delhi 2023-24, Ch. 13 (Govt of NCT Delhi, 2024): Domestic tariff w.e.f. 01.02.2018: up to 20 kL ₹5.27/kL, 20-30 ₹26.36, &gt;30 ₹43.93 plus 60% sewer charge; non-domestic &gt;100 kL ₹175.69/kL https://delhiplanning.delhi.gov.in/sites/default/files/Planning/chapter_13.pdf</t>
+          <t>KERC generic tariff for solar projects (1 Jul 2025 - 30 Jun 2026) (KERC, 2025): MW-scale solar benchmark tariff ₹3.04/unit; solar with battery storage ₹5.66/unit https://kerc.karnataka.gov.in/uploads/media_to_upload1752057190.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="11" t="inlineStr">
         <is>
-          <t>b3_rate</t>
+          <t>fixed_charge</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
@@ -12592,21 +12817,21 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Third block: rate</t>
+          <t>Fixed charge per connection</t>
         </is>
       </c>
       <c r="D77" s="11" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E77" s="11" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="F77" s="11" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="G77" s="11" t="inlineStr">
         <is>
-          <t>₹/kL</t>
+          <t>₹/connection/month</t>
         </is>
       </c>
       <c r="H77" s="11" t="inlineStr">
@@ -12616,34 +12841,39 @@
       </c>
       <c r="I77" s="11" t="inlineStr">
         <is>
-          <t>Discretionary use should pay the full financial cost, including replacing pipes and plants and paying for capital. The model puts that at about ₹104 per kL billed; Biome's S. Vishwanath estimated ₹95.</t>
+          <t>Much of a water system's cost is fixed, so many utilities charge a monthly fee per connection on top of the per-kilolitre rate. ₹100 is close to what Delhi charges and what BWSSB already collects as meter charges.</t>
         </is>
       </c>
       <c r="J77" s="11" t="inlineStr">
         <is>
-          <t>Comparators: BWSSB's bulk and non-domestic top rate is ₹99/kL; its own Sanchari Cauvery tanker sells 12 kL for ₹1,290 (≈₹107/kL).</t>
+          <t>BWSSB's meter charge today runs ₹30-150/month by slab; Delhi's service charge is ₹146.41 up to 20 kL. A high fixed charge falls hardest on small users, which is why it is kept modest.</t>
         </is>
       </c>
       <c r="K77" s="11" t="inlineStr">
         <is>
-          <t>Should Bengalureans really worry about the Cauvery water tariff hike? (Citizen Matters, 2025): S. Vishwanath: true cost of supply plus sewerage about ₹95/kL; 'nearly ₹40/kL to treat wastewater' https://citizenmatters.in/should-bengalureans-really-worry-about-the-cauvery-water-tariff-hike/</t>
+          <t>Revised Water Tariff Ready Reckoner 2025 (BWSSB, 2025): Domestic: 0-8 kL ₹8.5 (min ₹68), 8-25 ₹14, 25-50 ₹34, &gt;50 ₹55; sanitary ₹14 flat up to 8 kL; meter charge ₹30/50/75/150; bulk ₹99/kL; 3% auto increase each 1 April https://bwssb.karnataka.gov.in/storage/pdf-files/WaterTariff-2025.pdf</t>
         </is>
       </c>
       <c r="L77" s="11" t="inlineStr">
         <is>
-          <t>Revised Water Tariff Ready Reckoner 2025 (BWSSB, 2025): Domestic: 0-8 kL ₹8.5 (min ₹68), 8-25 ₹14, 25-50 ₹34, &gt;50 ₹55; sanitary ₹14 flat up to 8 kL; meter charge ₹30/50/75/150; bulk ₹99/kL; 3% auto increase each 1 April https://bwssb.karnataka.gov.in/storage/pdf-files/WaterTariff-2025.pdf</t>
+          <t>Water tariff (Delhi Jal Board, 2026): Domestic service charge ₹146.41/month up to 20 kL (₹219.62 for 20-30 kL, ₹292.82 above 30); free up to 20 kL with a functional meter; above 20 kL full consumption billed https://delhijalboard.delhi.gov.in/jalboard/about-us</t>
         </is>
       </c>
       <c r="M77" s="11" t="inlineStr">
         <is>
-          <t>BWSSB launches Sanchari Cauvery initiative (The Hindu, 2025): BWSSB tanker: 6 kL ₹740, 12 kL ₹1,290 within 2 km (≈ ₹107/kL) https://www.thehindu.com/news/cities/bangalore/amidst-rising-water-tanker-prices-bwssb-launches-sanchari-cauvery-initiative/article69557670.ece</t>
+          <t>Pricing Water Resources and Water and Sanitation Services (OECD, 2010): Countries are moving to 'two-part tariffs combining fixed charges and variable fees'; large share of fixed costs 'would call for their recovery through fixed charges' https://www.oecd.org/content/dam/oecd/en/publications/reports/2010/03/pricing-water-resources-and-water-and-sanitation-services_g1ghc680/9789264083608-en.pdf</t>
+        </is>
+      </c>
+      <c r="N77" s="11" t="inlineStr">
+        <is>
+          <t>Addressing the social consequences of tariffs for water supply and sanitation (OECD, 2020): Financial sustainability 'is likely to be strengthened if the tariff also includes a recurrent fixed charge', but fixed charges may raise social issues https://one.oecd.org/document/ENV/WKP(2020)13/En/pdf</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>b4_rate</t>
+          <t>b1_top</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
@@ -12653,21 +12883,21 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Top block: rate</t>
+          <t>Lifeline block: upper limit</t>
         </is>
       </c>
       <c r="D78" s="11" t="n">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="E78" s="11" t="n">
-        <v>110</v>
+        <v>8</v>
       </c>
       <c r="F78" s="11" t="n">
-        <v>220</v>
+        <v>15</v>
       </c>
       <c r="G78" s="11" t="inlineStr">
         <is>
-          <t>₹/kL</t>
+          <t>kL/month</t>
         </is>
       </c>
       <c r="H78" s="11" t="inlineStr">
@@ -12677,34 +12907,39 @@
       </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>The heaviest users should face the cost of bringing in the next source and the harm the system does. ₹150 a kL is about what a private water tanker charges in Bengaluru.</t>
+          <t>The first block should cover essential use at a low price. 10 kL a month is about 83 litres per person per day for a family of four: above WHO's 50-litre basic level, below the 135-litre planning norm.</t>
         </is>
       </c>
       <c r="J78" s="11" t="inlineStr">
         <is>
-          <t>Private 12 kL tankers: ₹1,600-1,800 (₹133-150/kL), up to ₹2,500 (₹208/kL). Delhi charges non-domestic users ₹175.69/kL above 100 kL; New York's water-only rate is ≈₹180/kL. The model's full economic cost is ~₹113/kL and full social cost ~₹189/kL.</t>
+          <t>4 × 50 L × 30 = 6 kL (WHO intermediate access); 4 × 100 L × 30 = 12 kL (top of OHCHR's 50-100 L); 4 × 135 L × 30 = 16.2 kL (CPHEEO). BWSSB's first slab is 8 kL; Delhi and Hyderabad give 20 kL free.</t>
         </is>
       </c>
       <c r="K78" s="11" t="inlineStr">
         <is>
-          <t>Long-term MoUs between Sanchari Cauvery and apartments (The Hindu, 2026): Private 12 kL tanker ₹1,600-1,800, touching ₹2,500 (≈ ₹133-208/kL); Sanchari ~₹1,300 https://www.thehindu.com/news/national/karnataka/long-term-mous-between-sanchari-cauvery-apartments-to-counter-skyrocketing-water-tanker-prices/article71278092.ece</t>
+          <t>Domestic water quantity, service level and health (2nd ed.) (WHO, 2020): Intermediate access: average quantity about 50 L/person/day; optimal access (multiple taps) 100+ L https://www.who.int/publications/i/item/9789240015241</t>
         </is>
       </c>
       <c r="L78" s="11" t="inlineStr">
         <is>
-          <t>Economic Survey of Delhi 2023-24, Ch. 13 (Govt of NCT Delhi, 2024): Domestic tariff w.e.f. 01.02.2018: up to 20 kL ₹5.27/kL, 20-30 ₹26.36, &gt;30 ₹43.93 plus 60% sewer charge; non-domestic &gt;100 kL ₹175.69/kL https://delhiplanning.delhi.gov.in/sites/default/files/Planning/chapter_13.pdf</t>
+          <t>FAQ on the human right to water and sanitation (OHCHR, 2012): 20 L/person/day is a minimum; 'States should aim for at least 50 to 100 litres per person per day' https://www.ohchr.org/sites/default/files/Documents/Issues/Water/FAQWater_en.pdf</t>
         </is>
       </c>
       <c r="M78" s="11" t="inlineStr">
         <is>
-          <t>FY2027 water and wastewater rate schedule (NYC Water Board, 2026): Water $5.35 per 100 cu ft (≈ $1.89/m³ ≈ ₹180/kL); sewer 159% of water https://www.nyc.gov/assets/nycwaterboard/downloads/pdf/rates/fy2027_rates.pdf</t>
+          <t>Handbook on Service Level Benchmarking (MoUD (now MoHUA), 2010): Per capita supply of water: benchmark 135 lpcd https://mohua.gov.in/static/uploads/2025/10/627238a27786db8ce624ea6c3db6ae24.pdf</t>
+        </is>
+      </c>
+      <c r="N78" s="11" t="inlineStr">
+        <is>
+          <t>Revised Water Tariff Ready Reckoner 2025 (BWSSB, 2025): Domestic: 0-8 kL ₹8.5 (min ₹68), 8-25 ₹14, 25-50 ₹34, &gt;50 ₹55; sanitary ₹14 flat up to 8 kL; meter charge ₹30/50/75/150; bulk ₹99/kL; 3% auto increase each 1 April https://bwssb.karnataka.gov.in/storage/pdf-files/WaterTariff-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="11" t="inlineStr">
         <is>
-          <t>connections_lakh</t>
+          <t>b1_rate</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
@@ -12714,478 +12949,844 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Water connections</t>
+          <t>Lifeline block: rate (all-in)</t>
         </is>
       </c>
       <c r="D79" s="11" t="n">
-        <v>11.3</v>
+        <v>15</v>
       </c>
       <c r="E79" s="11" t="n">
-        <v>10.7</v>
+        <v>8</v>
       </c>
       <c r="F79" s="11" t="n">
-        <v>11.5</v>
+        <v>25</v>
       </c>
       <c r="G79" s="11" t="inlineStr">
         <is>
-          <t>lakh</t>
+          <t>₹/kL</t>
         </is>
       </c>
       <c r="H79" s="11" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>Used to size the lifeline subsidy. BWSSB had more than 11.3 lakh connections in September 2026, up from 10.7 lakh in July 2024 as Stage V connections were added.</t>
-        </is>
-      </c>
-      <c r="J79" s="11" t="inlineStr"/>
+          <t>Today a household using 8 kL pays about ₹14.3 per kL all-in (water, sanitary and meter charges). Keeping the lifeline near that level protects the poorest from any increase.</t>
+        </is>
+      </c>
+      <c r="J79" s="11" t="inlineStr">
+        <is>
+          <t>FY27 bill at 8 kL: minimum ₹68 × 1.03 + sanitary ₹14 × 1.03 + meter ₹30 = ₹114.5 ÷ 8 = ₹14.3/kL. Chennai charges ₹8/kL up to 10 kL; Hyderabad ~₹10/kL with 20 kL free.</t>
+        </is>
+      </c>
       <c r="K79" s="11" t="inlineStr">
         <is>
-          <t>BWSSB's ₹4.87 crore plan aims to cut household water use (Bangalore Mirror, 2026): More than 11.3 lakh connections https://bangaloremirror.indiatimes.com/bangalore/others/bwssbs-rs-4-87-crore-plan-aims-to-cut-household-water-use-by-up-to-25/articleshow/133812045.cms</t>
+          <t>Revised Water Tariff Ready Reckoner 2025 (BWSSB, 2025): Domestic: 0-8 kL ₹8.5 (min ₹68), 8-25 ₹14, 25-50 ₹34, &gt;50 ₹55; sanitary ₹14 flat up to 8 kL; meter charge ₹30/50/75/150; bulk ₹99/kL; 3% auto increase each 1 April https://bwssb.karnataka.gov.in/storage/pdf-files/WaterTariff-2025.pdf</t>
         </is>
       </c>
       <c r="L79" s="11" t="inlineStr">
         <is>
-          <t>Presentation by Chief Engineer, BWSSB (BWSSB (via AMDA), 2024): 10.70 lakh house connections; 9.70 lakh sanitary connections https://amdaindia.org/wp-content/uploads/Presentation-by-Chief-Engineer-Bangalore-Water-Supply-and-Sewerage-Board-WATER-SENSITIVITY-MS-3rd-PPT-Part-II.pdf</t>
+          <t>Water and sewerage tariff (CMWSSB (Chennai), 2026): Domestic: up to 10 kL ₹8/kL, 11-15 ₹20, 16-25 ₹32, above 25 ₹51; minimum ₹111/month incl. sewer https://cmwssb.tn.gov.in/tariff</t>
         </is>
       </c>
       <c r="M79" s="11" t="inlineStr">
         <is>
-          <t>Cauvery in the pipeline, but 110 villages have connection problems (The Hindu, 2024): About 10.6 lakh connections, October 2024 https://www.thehindu.com/news/cities/bangalore/cauvery-in-the-pipeline-but-110-villages-on-bengalurus-outskirts-have-connection-problems/article68701995.ece</t>
+          <t>Water bills set to rise 5% every year as HMWSSB seeks to plug revenue gap (Times of India, 2026): Tariff about ₹10/kL; 20 kL free for about 5 lakh households; 5% annual hike https://timesofindia.indiatimes.com/city/hyderabad/water-bills-set-to-rise-5-every-yr-as-hmwssb-seeks-to-plug-revenue-gap/articleshow/134291436.cms</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>hh_size</t>
+          <t>b2_top</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Persons per household, Bengaluru</t>
+          <t>Second block: upper limit</t>
         </is>
       </c>
       <c r="D80" s="11" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E80" s="11" t="n">
-        <v>3.5</v>
+        <v>15</v>
       </c>
       <c r="F80" s="11" t="n">
-        <v>4.5</v>
+        <v>30</v>
       </c>
       <c r="G80" s="11" t="inlineStr">
         <is>
-          <t>persons</t>
+          <t>kL/month</t>
         </is>
       </c>
       <c r="H80" s="11" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>The 2011 Census counted about 4.0 people per household in Bengaluru. Urban households have been shrinking since, so the range runs down to 3.5.</t>
+          <t>The second block covers ordinary family use up to the planning norm. A family of four at 135-150 litres a day uses 16-18 kL a month.</t>
         </is>
       </c>
       <c r="J80" s="11" t="inlineStr">
         <is>
-          <t>NFHS-5 (2019-21) found 4.2 per household for Karnataka and 4.4 for India; a Bengaluru city figure exists in NFHS-5 CSVs on OpenCity but was not extracted.</t>
+          <t>4 × 135 × 30 = 16.2 kL; 4 × 150 × 30 = 18 kL. Delhi's tariff steps at 20 and 30 kL.</t>
         </is>
       </c>
       <c r="K80" s="11" t="inlineStr">
         <is>
-          <t>BBMP city population, Census 2011 (Census of India (via censusindia2011.com), 2011): 8,443,675 people in 2,101,831 households → 4.02 https://www.censusindia2011.com/karnataka/bangalore/no-sub-district/bbmp-m-corp-part-population.html</t>
+          <t>Handbook on Service Level Benchmarking (MoUD (now MoHUA), 2010): Per capita supply of water: benchmark 135 lpcd https://mohua.gov.in/static/uploads/2025/10/627238a27786db8ce624ea6c3db6ae24.pdf</t>
         </is>
       </c>
       <c r="L80" s="11" t="inlineStr">
         <is>
-          <t>Bengaluru Urban district (villageinfo.in (Census 2011), 2011): 23,93,845 households in Bengaluru Urban district https://villageinfo.in/karnataka/bengaluru-urban/</t>
+          <t>CPHEEO Manual on Water Supply and Treatment (copy) (CPHEEO (Scribd copy), 1999): 135 lpcd for cities with sewerage; 150 lpcd for metropolitan and mega cities https://www.scribd.com/document/813009957/CPHEEO-Manual-on-Water-Supply</t>
         </is>
       </c>
       <c r="M80" s="11" t="inlineStr">
         <is>
-          <t>Bengaluru Urban district (Wikipedia (Census 2011), 2011): Population 9,621,551 → 4.02 per household with the count above https://en.wikipedia.org/wiki/Bengaluru_Urban_district</t>
+          <t>Water tariff (Delhi Jal Board, 2026): Domestic service charge ₹146.41/month up to 20 kL (₹219.62 for 20-30 kL, ₹292.82 above 30); free up to 20 kL with a functional meter; above 20 kL full consumption billed https://delhijalboard.delhi.gov.in/jalboard/about-us</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="11" t="inlineStr">
         <is>
-          <t>lpcd_norm</t>
+          <t>b2_rate</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Water each person needs (CPHEEO norm)</t>
+          <t>Second block: rate</t>
         </is>
       </c>
       <c r="D81" s="11" t="n">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="E81" s="11" t="n">
-        <v>108</v>
+        <v>40</v>
       </c>
       <c r="F81" s="11" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="G81" s="11" t="inlineStr">
         <is>
-          <t>litres/person/day</t>
+          <t>₹/kL</t>
         </is>
       </c>
       <c r="H81" s="11" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>India's planning norm is 135 litres per person per day for cities with sewers, and 150 for metros. Bengaluru's own average is 108.</t>
+          <t>Normal household use should at least pay what it costs BWSSB to run the system today. BWSSB itself says it spends about ₹54 per kL; the model's cash cost per kL billed is about ₹62.</t>
         </is>
       </c>
       <c r="J81" s="11" t="inlineStr">
         <is>
-          <t>At 4 people × 135 lpcd × 30 days, a household uses about 16 kL a month.</t>
+          <t>Comparators: Chennai charges ₹51/kL above 25 kL; Delhi ₹26.36/kL (20-30 kL) plus 60% sewer = ₹42/kL plus service charge. ₹60 is roughly 4× today's ₹14/kL second slab.</t>
         </is>
       </c>
       <c r="K81" s="11" t="inlineStr">
         <is>
-          <t>Handbook on Service Level Benchmarking (MoUD (now MoHUA), 2010): Per capita supply of water: benchmark 135 lpcd https://mohua.gov.in/static/uploads/2025/10/627238a27786db8ce624ea6c3db6ae24.pdf</t>
+          <t>Water supply to core city ramped up (chairman interview) (New Indian Express, 2026): 'BWSSB spends around ₹54 per 1,000 litres to draw, treat and supply Cauvery water'; households pay ₹20-30/kL on average https://www.newindianexpress.com/cities/bengaluru/2026/May/18/water-supply-to-core-city-ramped-up-pipeline-network-for-suburbs-under-way-bwssb-chairman</t>
         </is>
       </c>
       <c r="L81" s="11" t="inlineStr">
         <is>
-          <t>Per capita availability of water (Rajya Sabha reply) (PIB / Ministry of Jal Shakti, 2020): MoHUA suggests 135 lpcd as the urban benchmark https://www.pib.gov.in/PressReleasePage.aspx?PRID=1604871</t>
+          <t>Water and sewerage tariff (CMWSSB (Chennai), 2026): Domestic: up to 10 kL ₹8/kL, 11-15 ₹20, 16-25 ₹32, above 25 ₹51; minimum ₹111/month incl. sewer https://cmwssb.tn.gov.in/tariff</t>
         </is>
       </c>
       <c r="M81" s="11" t="inlineStr">
         <is>
-          <t>CPHEEO Manual on Water Supply and Treatment (copy) (CPHEEO (Scribd copy), 1999): 135 lpcd for cities with sewerage; 150 lpcd for metropolitan and mega cities https://www.scribd.com/document/813009957/CPHEEO-Manual-on-Water-Supply</t>
-        </is>
-      </c>
-      <c r="N81" s="11" t="inlineStr">
-        <is>
-          <t>Presentation by Chief Engineer, BWSSB (BWSSB (via AMDA), 2024): Average per capita consumption 108 L/day https://amdaindia.org/wp-content/uploads/Presentation-by-Chief-Engineer-Bangalore-Water-Supply-and-Sewerage-Board-WATER-SENSITIVITY-MS-3rd-PPT-Part-II.pdf</t>
+          <t>Economic Survey of Delhi 2023-24, Ch. 13 (Govt of NCT Delhi, 2024): Domestic tariff w.e.f. 01.02.2018: up to 20 kL ₹5.27/kL, 20-30 ₹26.36, &gt;30 ₹43.93 plus 60% sewer charge; non-domestic &gt;100 kL ₹175.69/kL https://delhiplanning.delhi.gov.in/sites/default/files/Planning/chapter_13.pdf</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>hh_income_low</t>
+          <t>b3_top</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Lower-income household income</t>
+          <t>Third block: upper limit</t>
         </is>
       </c>
       <c r="D82" s="11" t="n">
-        <v>25000</v>
+        <v>40</v>
       </c>
       <c r="E82" s="11" t="n">
-        <v>15000</v>
+        <v>30</v>
       </c>
       <c r="F82" s="11" t="n">
-        <v>35000</v>
+        <v>60</v>
       </c>
       <c r="G82" s="11" t="inlineStr">
         <is>
-          <t>₹/month</t>
+          <t>kL/month</t>
         </is>
       </c>
       <c r="H82" s="11" t="inlineStr">
         <is>
-          <t>assumed</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>Karnataka's May 2026 minimum wage for unskilled work in Bengaluru is ₹23,376 a month. A household with one such earner, plus a little extra, has about ₹25,000.</t>
+          <t>Above about 40 kL a month a household is watering gardens or filling tanks, which is discretionary use. BWSSB's own third slab runs 25-50 kL.</t>
         </is>
       </c>
       <c r="J82" s="11" t="inlineStr">
         <is>
-          <t>The notification is being challenged in the High Court, and many informal workers earn below it; the low end (₹15,000) reflects that. No survey-based Bengaluru income distribution was found.</t>
+          <t>40 kL is more than twice the 18 kL a family of four needs at 150 lpcd. Delhi's top slab starts at 30 kL.</t>
         </is>
       </c>
       <c r="K82" s="11" t="inlineStr">
         <is>
-          <t>Karnataka hikes minimum wages in 81 sectors by 60% (New Indian Express, 2026): Zone-1 Bengaluru unskilled ₹23,376/month; highly skilled ₹31,114 https://www.newindianexpress.com/story/states/karnataka/2026/may/24/karnataka-hikes-minimum-wages-in-81-sectors-by-60</t>
+          <t>Revised Water Tariff Ready Reckoner 2025 (BWSSB, 2025): Domestic: 0-8 kL ₹8.5 (min ₹68), 8-25 ₹14, 25-50 ₹34, &gt;50 ₹55; sanitary ₹14 flat up to 8 kL; meter charge ₹30/50/75/150; bulk ₹99/kL; 3% auto increase each 1 April https://bwssb.karnataka.gov.in/storage/pdf-files/WaterTariff-2025.pdf</t>
         </is>
       </c>
       <c r="L82" s="11" t="inlineStr">
         <is>
-          <t>Karnataka notifies final minimum wages, average increase 60% (The Hindu, 2026): Final notification 22 May 2026: ₹19,300-31,100 per month https://www.thehindu.com/news/national/karnataka/karnataka-notifies-final-draft-of-minimum-wages-with-average-increase-of-60/article71011111.ece</t>
+          <t>CPHEEO Manual on Water Supply and Treatment (copy) (CPHEEO (Scribd copy), 1999): 135 lpcd for cities with sewerage; 150 lpcd for metropolitan and mega cities https://www.scribd.com/document/813009957/CPHEEO-Manual-on-Water-Supply</t>
         </is>
       </c>
       <c r="M82" s="11" t="inlineStr">
         <is>
-          <t>Single final notification on minimum wage rates (Karnataka Labour Department, 2026): Gazette text of the 22 May 2026 notification https://karmikaspandana.karnataka.gov.in/uploads/media_to_upload1780292271.pdf</t>
+          <t>Economic Survey of Delhi 2023-24, Ch. 13 (Govt of NCT Delhi, 2024): Domestic tariff w.e.f. 01.02.2018: up to 20 kL ₹5.27/kL, 20-30 ₹26.36, &gt;30 ₹43.93 plus 60% sewer charge; non-domestic &gt;100 kL ₹175.69/kL https://delhiplanning.delhi.gov.in/sites/default/files/Planning/chapter_13.pdf</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="11" t="inlineStr">
         <is>
-          <t>hh_income_mid</t>
+          <t>b3_rate</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Middle-income household income</t>
+          <t>Third block: rate</t>
         </is>
       </c>
       <c r="D83" s="11" t="n">
-        <v>75000</v>
+        <v>105</v>
       </c>
       <c r="E83" s="11" t="n">
-        <v>42000</v>
+        <v>90</v>
       </c>
       <c r="F83" s="11" t="n">
-        <v>125000</v>
+        <v>130</v>
       </c>
       <c r="G83" s="11" t="inlineStr">
         <is>
-          <t>₹/month</t>
+          <t>₹/kL</t>
         </is>
       </c>
       <c r="H83" s="11" t="inlineStr">
         <is>
-          <t>assumed</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="I83" s="11" t="inlineStr">
         <is>
-          <t>₹75,000 a month (₹9 lakh a year) is a typical middle-class Bengaluru household. It sits in PRICE's 'seeker' band of ₹5-15 lakh a year, well below the city's skewed average of ₹28 lakh.</t>
+          <t>Discretionary use should pay the full financial cost, including replacing pipes and plants and paying for capital. The model puts that at about ₹104 per kL billed; Biome's S. Vishwanath estimated ₹95.</t>
         </is>
       </c>
       <c r="J83" s="11" t="inlineStr">
         <is>
-          <t>The ₹28 lakh figure is a mean pulled up by high earners; a median was not found. The range ₹42,000-1,25,000/month is the seeker band in 2020-21 rupees.</t>
+          <t>Comparators: BWSSB's bulk and non-domestic top rate is ₹99/kL; its own Sanchari Cauvery tanker sells 12 kL for ₹1,290 (≈₹107/kL).</t>
         </is>
       </c>
       <c r="K83" s="11" t="inlineStr">
         <is>
-          <t>India's Middle Class: executive summary (ICE 360) (PRICE, 2023): Middle class ₹5-30 lakh/yr household income; 'seekers' ₹5-15 lakh (2020-21 prices) https://price360.in/Executive_Summary_Middle_Class.pdf</t>
+          <t>Should Bengalureans really worry about the Cauvery water tariff hike? (Citizen Matters, 2025): S. Vishwanath: true cost of supply plus sewerage about ₹95/kL; 'nearly ₹40/kL to treat wastewater' https://citizenmatters.in/should-bengalureans-really-worry-about-the-cauvery-water-tariff-hike/</t>
         </is>
       </c>
       <c r="L83" s="11" t="inlineStr">
         <is>
-          <t>Bengaluru, Chandigarh pip Mumbai, Delhi in average household income (Business Standard, 2026): Bengaluru average household income ₹28.3 lakh/yr (FY25-26, PRICE with Tata Sons) https://www.business-standard.com/finance/personal-finance/bengaluru-chandigarh-pip-mumbai-delhi-in-average-household-income-study-126071300629_1.html</t>
+          <t>Revised Water Tariff Ready Reckoner 2025 (BWSSB, 2025): Domestic: 0-8 kL ₹8.5 (min ₹68), 8-25 ₹14, 25-50 ₹34, &gt;50 ₹55; sanitary ₹14 flat up to 8 kL; meter charge ₹30/50/75/150; bulk ₹99/kL; 3% auto increase each 1 April https://bwssb.karnataka.gov.in/storage/pdf-files/WaterTariff-2025.pdf</t>
         </is>
       </c>
       <c r="M83" s="11" t="inlineStr">
         <is>
-          <t>Metros dominate incomes (The Many Urban Indias) (Moneycontrol, 2026): Bengaluru and Chandigarh highest average household income, ~₹28 lakh/yr https://www.moneycontrol.com/news/business/economy/metros-dominate-incomes-but-tiruppur-and-surat-outshine-in-household-spending-price-report-13965832.html</t>
+          <t>BWSSB launches Sanchari Cauvery initiative (The Hindu, 2025): BWSSB tanker: 6 kL ₹740, 12 kL ₹1,290 within 2 km (≈ ₹107/kL) https://www.thehindu.com/news/cities/bangalore/amidst-rising-water-tanker-prices-bwssb-launches-sanchari-cauvery-initiative/article69557670.ece</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>afford_pct</t>
+          <t>b4_rate</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Affordability threshold (share of income)</t>
+          <t>Top block: rate</t>
         </is>
       </c>
       <c r="D84" s="11" t="n">
-        <v>0.03</v>
+        <v>150</v>
       </c>
       <c r="E84" s="11" t="n">
-        <v>0.03</v>
+        <v>110</v>
       </c>
       <c r="F84" s="11" t="n">
-        <v>0.05</v>
+        <v>220</v>
       </c>
       <c r="G84" s="11" t="inlineStr">
         <is>
-          <t>share of income</t>
+          <t>₹/kL</t>
         </is>
       </c>
       <c r="H84" s="11" t="inlineStr">
         <is>
-          <t>sourced</t>
+          <t>policy</t>
         </is>
       </c>
       <c r="I84" s="11" t="inlineStr">
         <is>
-          <t>The UN suggests a household should not spend more than about 3% of its income on water; World Bank work uses up to 5%. Above that, water is unaffordable.</t>
-        </is>
-      </c>
-      <c r="J84" s="11" t="inlineStr"/>
+          <t>The heaviest users should face the cost of bringing in the next source and the harm the system does. ₹150 a kL is about what a private water tanker charges in Bengaluru.</t>
+        </is>
+      </c>
+      <c r="J84" s="11" t="inlineStr">
+        <is>
+          <t>Private 12 kL tankers: ₹1,600-1,800 (₹133-150/kL), up to ₹2,500 (₹208/kL). Delhi charges non-domestic users ₹175.69/kL above 100 kL; New York's water-only rate is ≈₹180/kL. The model's full economic cost is ~₹113/kL and full social cost ~₹189/kL.</t>
+        </is>
+      </c>
       <c r="K84" s="11" t="inlineStr">
         <is>
-          <t>Human Development Report 2006 (summary) (UNDP, 2006): Target ceiling of 3% for the share of household income spent on water https://hdr.undp.org/system/files/documents/human-development-report-2006-summary-english.human-development-report-2006-summary-english</t>
+          <t>Long-term MoUs between Sanchari Cauvery and apartments (The Hindu, 2026): Private 12 kL tanker ₹1,600-1,800, touching ₹2,500 (≈ ₹133-208/kL); Sanchari ~₹1,300 https://www.thehindu.com/news/national/karnataka/long-term-mous-between-sanchari-cauvery-apartments-to-counter-skyrocketing-water-tanker-prices/article71278092.ece</t>
         </is>
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>Human Development Report 2006 (full report) (UNDP, 2006): Cites Foster &amp; Yepes (World Bank) defining affordability as water at most 5% of income https://files.acquia.undp.org/public/migration/tr/HDR06-complete.pdf</t>
+          <t>Economic Survey of Delhi 2023-24, Ch. 13 (Govt of NCT Delhi, 2024): Domestic tariff w.e.f. 01.02.2018: up to 20 kL ₹5.27/kL, 20-30 ₹26.36, &gt;30 ₹43.93 plus 60% sewer charge; non-domestic &gt;100 kL ₹175.69/kL https://delhiplanning.delhi.gov.in/sites/default/files/Planning/chapter_13.pdf</t>
         </is>
       </c>
       <c r="M84" s="11" t="inlineStr">
         <is>
-          <t>Pricing Water Resources and Water and Sanitation Services (OECD, 2010): No official threshold; Portugal's regulator used 3% of disposable income https://www.oecd.org/content/dam/oecd/en/publications/reports/2010/03/pricing-water-resources-and-water-and-sanitation-services_g1ghc680/9789264083608-en.pdf</t>
-        </is>
-      </c>
-      <c r="N84" s="11" t="inlineStr">
-        <is>
-          <t>Water Affordability Needs Assessment (US EPA, 2024): Uses 3% and 4.5% of household income for water + wastewater https://www.epa.gov/waterfinancecenter/water-affordability-needs-assessment</t>
+          <t>FY2027 water and wastewater rate schedule (NYC Water Board, 2026): Water $5.35 per 100 cu ft (≈ $1.89/m³ ≈ ₹180/kL); sewer 159% of water https://www.nyc.gov/assets/nycwaterboard/downloads/pdf/rates/fy2027_rates.pdf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="11" t="inlineStr">
         <is>
-          <t>tanker_rs_kl</t>
+          <t>connections_lakh</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Households and affordability</t>
+          <t>A tariff that would work</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Private tanker water price (2025-26)</t>
+          <t>Water connections</t>
         </is>
       </c>
       <c r="D85" s="11" t="n">
-        <v>140</v>
+        <v>11.3</v>
       </c>
       <c r="E85" s="11" t="n">
-        <v>115</v>
+        <v>10.7</v>
       </c>
       <c r="F85" s="11" t="n">
-        <v>210</v>
+        <v>11.5</v>
       </c>
       <c r="G85" s="11" t="inlineStr">
         <is>
-          <t>₹/kL</t>
+          <t>lakh</t>
         </is>
       </c>
       <c r="H85" s="11" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>sourced</t>
         </is>
       </c>
       <c r="I85" s="11" t="inlineStr">
         <is>
-          <t>A 12,000-litre private tanker costs ₹1,600-1,800 in 2026, about ₹140 per kL, and up to ₹2,500 in bad weeks. That is several times the piped tariff.</t>
-        </is>
-      </c>
-      <c r="J85" s="11" t="inlineStr">
-        <is>
-          <t>₹/kL is our arithmetic: ₹1,700 ÷ 12 kL ≈ ₹142. In the 2024 crisis, 6 kL went for up to ₹3,000 (₹500/kL).</t>
-        </is>
-      </c>
+          <t>Used to size the lifeline subsidy. BWSSB had more than 11.3 lakh connections in September 2026, up from 10.7 lakh in July 2024 as Stage V connections were added.</t>
+        </is>
+      </c>
+      <c r="J85" s="11" t="inlineStr"/>
       <c r="K85" s="11" t="inlineStr">
         <is>
-          <t>Long-term MoUs between Sanchari Cauvery and apartments (The Hindu, 2026): Private 12 kL ₹1,600-1,800, touching ₹2,500 https://www.thehindu.com/news/national/karnataka/long-term-mous-between-sanchari-cauvery-apartments-to-counter-skyrocketing-water-tanker-prices/article71278092.ece</t>
+          <t>BWSSB's ₹4.87 crore plan aims to cut household water use (Bangalore Mirror, 2026): More than 11.3 lakh connections https://bangaloremirror.indiatimes.com/bangalore/others/bwssbs-rs-4-87-crore-plan-aims-to-cut-household-water-use-by-up-to-25/articleshow/133812045.cms</t>
         </is>
       </c>
       <c r="L85" s="11" t="inlineStr">
         <is>
-          <t>Residents struggle to pay soaring water tanker costs (Deccan Herald, 2025): 6 kL ₹600-650; 12 kL ~₹1,400 https://www.deccanherald.com/india/karnataka/bengaluru/heat-burns-the-pocket-residents-struggle-to-pay-soaring-water-tanker-costs-3450484</t>
+          <t>Presentation by Chief Engineer, BWSSB (BWSSB (via AMDA), 2024): 10.70 lakh house connections; 9.70 lakh sanitary connections https://amdaindia.org/wp-content/uploads/Presentation-by-Chief-Engineer-Bangalore-Water-Supply-and-Sewerage-Board-WATER-SENSITIVITY-MS-3rd-PPT-Part-II.pdf</t>
         </is>
       </c>
       <c r="M85" s="11" t="inlineStr">
         <is>
-          <t>Karnataka govt caps tanker water prices (New Indian Express, 2024): 2024 cap: 12 kL ₹1,000 (≤5 km) / ₹1,200 (5-10 km) https://www.newindianexpress.com/states/karnataka/2024/Mar/08/karnataka-govt-acts-caps-tanker-water-prices</t>
+          <t>Cauvery in the pipeline, but 110 villages have connection problems (The Hindu, 2024): About 10.6 lakh connections, October 2024 https://www.thehindu.com/news/cities/bangalore/cauvery-in-the-pipeline-but-110-villages-on-bengalurus-outskirts-have-connection-problems/article68701995.ece</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="11" t="inlineStr">
         <is>
+          <t>hh_size</t>
+        </is>
+      </c>
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+      <c r="C86" s="11" t="inlineStr">
+        <is>
+          <t>Persons per household, Bengaluru</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E86" s="11" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F86" s="11" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G86" s="11" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="H86" s="11" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="I86" s="11" t="inlineStr">
+        <is>
+          <t>The 2011 Census counted about 4.0 people per household in Bengaluru. Urban households have been shrinking since, so the range runs down to 3.5.</t>
+        </is>
+      </c>
+      <c r="J86" s="11" t="inlineStr">
+        <is>
+          <t>NFHS-5 (2019-21) found 4.2 per household for Karnataka and 4.4 for India; a Bengaluru city figure exists in NFHS-5 CSVs on OpenCity but was not extracted.</t>
+        </is>
+      </c>
+      <c r="K86" s="11" t="inlineStr">
+        <is>
+          <t>BBMP city population, Census 2011 (Census of India (via censusindia2011.com), 2011): 8,443,675 people in 2,101,831 households → 4.02 https://www.censusindia2011.com/karnataka/bangalore/no-sub-district/bbmp-m-corp-part-population.html</t>
+        </is>
+      </c>
+      <c r="L86" s="11" t="inlineStr">
+        <is>
+          <t>Bengaluru Urban district (villageinfo.in (Census 2011), 2011): 23,93,845 households in Bengaluru Urban district https://villageinfo.in/karnataka/bengaluru-urban/</t>
+        </is>
+      </c>
+      <c r="M86" s="11" t="inlineStr">
+        <is>
+          <t>Bengaluru Urban district (Wikipedia (Census 2011), 2011): Population 9,621,551 → 4.02 per household with the count above https://en.wikipedia.org/wiki/Bengaluru_Urban_district</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="11" t="inlineStr">
+        <is>
+          <t>lpcd_norm</t>
+        </is>
+      </c>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="inlineStr">
+        <is>
+          <t>Water each person needs (CPHEEO norm)</t>
+        </is>
+      </c>
+      <c r="D87" s="11" t="n">
+        <v>135</v>
+      </c>
+      <c r="E87" s="11" t="n">
+        <v>108</v>
+      </c>
+      <c r="F87" s="11" t="n">
+        <v>150</v>
+      </c>
+      <c r="G87" s="11" t="inlineStr">
+        <is>
+          <t>litres/person/day</t>
+        </is>
+      </c>
+      <c r="H87" s="11" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="I87" s="11" t="inlineStr">
+        <is>
+          <t>India's planning norm is 135 litres per person per day for cities with sewers, and 150 for metros. Bengaluru's own average is 108.</t>
+        </is>
+      </c>
+      <c r="J87" s="11" t="inlineStr">
+        <is>
+          <t>At 4 people × 135 lpcd × 30 days, a household uses about 16 kL a month.</t>
+        </is>
+      </c>
+      <c r="K87" s="11" t="inlineStr">
+        <is>
+          <t>Handbook on Service Level Benchmarking (MoUD (now MoHUA), 2010): Per capita supply of water: benchmark 135 lpcd https://mohua.gov.in/static/uploads/2025/10/627238a27786db8ce624ea6c3db6ae24.pdf</t>
+        </is>
+      </c>
+      <c r="L87" s="11" t="inlineStr">
+        <is>
+          <t>Per capita availability of water (Rajya Sabha reply) (PIB / Ministry of Jal Shakti, 2020): MoHUA suggests 135 lpcd as the urban benchmark https://www.pib.gov.in/PressReleasePage.aspx?PRID=1604871</t>
+        </is>
+      </c>
+      <c r="M87" s="11" t="inlineStr">
+        <is>
+          <t>CPHEEO Manual on Water Supply and Treatment (copy) (CPHEEO (Scribd copy), 1999): 135 lpcd for cities with sewerage; 150 lpcd for metropolitan and mega cities https://www.scribd.com/document/813009957/CPHEEO-Manual-on-Water-Supply</t>
+        </is>
+      </c>
+      <c r="N87" s="11" t="inlineStr">
+        <is>
+          <t>Presentation by Chief Engineer, BWSSB (BWSSB (via AMDA), 2024): Average per capita consumption 108 L/day https://amdaindia.org/wp-content/uploads/Presentation-by-Chief-Engineer-Bangalore-Water-Supply-and-Sewerage-Board-WATER-SENSITIVITY-MS-3rd-PPT-Part-II.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="11" t="inlineStr">
+        <is>
+          <t>hh_income_low</t>
+        </is>
+      </c>
+      <c r="B88" s="11" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+      <c r="C88" s="11" t="inlineStr">
+        <is>
+          <t>Lower-income household income</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E88" s="11" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F88" s="11" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G88" s="11" t="inlineStr">
+        <is>
+          <t>₹/month</t>
+        </is>
+      </c>
+      <c r="H88" s="11" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="I88" s="11" t="inlineStr">
+        <is>
+          <t>Karnataka's May 2026 minimum wage for unskilled work in Bengaluru is ₹23,376 a month. A household with one such earner, plus a little extra, has about ₹25,000.</t>
+        </is>
+      </c>
+      <c r="J88" s="11" t="inlineStr">
+        <is>
+          <t>The notification is being challenged in the High Court, and many informal workers earn below it; the low end (₹15,000) reflects that. No survey-based Bengaluru income distribution was found.</t>
+        </is>
+      </c>
+      <c r="K88" s="11" t="inlineStr">
+        <is>
+          <t>Karnataka hikes minimum wages in 81 sectors by 60% (New Indian Express, 2026): Zone-1 Bengaluru unskilled ₹23,376/month; highly skilled ₹31,114 https://www.newindianexpress.com/story/states/karnataka/2026/may/24/karnataka-hikes-minimum-wages-in-81-sectors-by-60</t>
+        </is>
+      </c>
+      <c r="L88" s="11" t="inlineStr">
+        <is>
+          <t>Karnataka notifies final minimum wages, average increase 60% (The Hindu, 2026): Final notification 22 May 2026: ₹19,300-31,100 per month https://www.thehindu.com/news/national/karnataka/karnataka-notifies-final-draft-of-minimum-wages-with-average-increase-of-60/article71011111.ece</t>
+        </is>
+      </c>
+      <c r="M88" s="11" t="inlineStr">
+        <is>
+          <t>Single final notification on minimum wage rates (Karnataka Labour Department, 2026): Gazette text of the 22 May 2026 notification https://karmikaspandana.karnataka.gov.in/uploads/media_to_upload1780292271.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="11" t="inlineStr">
+        <is>
+          <t>hh_income_mid</t>
+        </is>
+      </c>
+      <c r="B89" s="11" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+      <c r="C89" s="11" t="inlineStr">
+        <is>
+          <t>Middle-income household income</t>
+        </is>
+      </c>
+      <c r="D89" s="11" t="n">
+        <v>75000</v>
+      </c>
+      <c r="E89" s="11" t="n">
+        <v>42000</v>
+      </c>
+      <c r="F89" s="11" t="n">
+        <v>125000</v>
+      </c>
+      <c r="G89" s="11" t="inlineStr">
+        <is>
+          <t>₹/month</t>
+        </is>
+      </c>
+      <c r="H89" s="11" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="I89" s="11" t="inlineStr">
+        <is>
+          <t>₹75,000 a month (₹9 lakh a year) is a typical middle-class Bengaluru household. It sits in PRICE's 'seeker' band of ₹5-15 lakh a year, well below the city's skewed average of ₹28 lakh.</t>
+        </is>
+      </c>
+      <c r="J89" s="11" t="inlineStr">
+        <is>
+          <t>The ₹28 lakh figure is a mean pulled up by high earners; a median was not found. The range ₹42,000-1,25,000/month is the seeker band in 2020-21 rupees.</t>
+        </is>
+      </c>
+      <c r="K89" s="11" t="inlineStr">
+        <is>
+          <t>India's Middle Class: executive summary (ICE 360) (PRICE, 2023): Middle class ₹5-30 lakh/yr household income; 'seekers' ₹5-15 lakh (2020-21 prices) https://price360.in/Executive_Summary_Middle_Class.pdf</t>
+        </is>
+      </c>
+      <c r="L89" s="11" t="inlineStr">
+        <is>
+          <t>Bengaluru, Chandigarh pip Mumbai, Delhi in average household income (Business Standard, 2026): Bengaluru average household income ₹28.3 lakh/yr (FY25-26, PRICE with Tata Sons) https://www.business-standard.com/finance/personal-finance/bengaluru-chandigarh-pip-mumbai-delhi-in-average-household-income-study-126071300629_1.html</t>
+        </is>
+      </c>
+      <c r="M89" s="11" t="inlineStr">
+        <is>
+          <t>Metros dominate incomes (The Many Urban Indias) (Moneycontrol, 2026): Bengaluru and Chandigarh highest average household income, ~₹28 lakh/yr https://www.moneycontrol.com/news/business/economy/metros-dominate-incomes-but-tiruppur-and-surat-outshine-in-household-spending-price-report-13965832.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>afford_pct</t>
+        </is>
+      </c>
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+      <c r="C90" s="11" t="inlineStr">
+        <is>
+          <t>Affordability threshold (share of income)</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E90" s="11" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F90" s="11" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G90" s="11" t="inlineStr">
+        <is>
+          <t>share of income</t>
+        </is>
+      </c>
+      <c r="H90" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="I90" s="11" t="inlineStr">
+        <is>
+          <t>The UN suggests a household should not spend more than about 3% of its income on water; World Bank work uses up to 5%. Above that, water is unaffordable.</t>
+        </is>
+      </c>
+      <c r="J90" s="11" t="inlineStr"/>
+      <c r="K90" s="11" t="inlineStr">
+        <is>
+          <t>Human Development Report 2006 (summary) (UNDP, 2006): Target ceiling of 3% for the share of household income spent on water https://hdr.undp.org/system/files/documents/human-development-report-2006-summary-english.human-development-report-2006-summary-english</t>
+        </is>
+      </c>
+      <c r="L90" s="11" t="inlineStr">
+        <is>
+          <t>Human Development Report 2006 (full report) (UNDP, 2006): Cites Foster &amp; Yepes (World Bank) defining affordability as water at most 5% of income https://files.acquia.undp.org/public/migration/tr/HDR06-complete.pdf</t>
+        </is>
+      </c>
+      <c r="M90" s="11" t="inlineStr">
+        <is>
+          <t>Pricing Water Resources and Water and Sanitation Services (OECD, 2010): No official threshold; Portugal's regulator used 3% of disposable income https://www.oecd.org/content/dam/oecd/en/publications/reports/2010/03/pricing-water-resources-and-water-and-sanitation-services_g1ghc680/9789264083608-en.pdf</t>
+        </is>
+      </c>
+      <c r="N90" s="11" t="inlineStr">
+        <is>
+          <t>Water Affordability Needs Assessment (US EPA, 2024): Uses 3% and 4.5% of household income for water + wastewater https://www.epa.gov/waterfinancecenter/water-affordability-needs-assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="11" t="inlineStr">
+        <is>
+          <t>tanker_rs_kl</t>
+        </is>
+      </c>
+      <c r="B91" s="11" t="inlineStr">
+        <is>
+          <t>Households and affordability</t>
+        </is>
+      </c>
+      <c r="C91" s="11" t="inlineStr">
+        <is>
+          <t>Private tanker water price (2025-26)</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="n">
+        <v>140</v>
+      </c>
+      <c r="E91" s="11" t="n">
+        <v>115</v>
+      </c>
+      <c r="F91" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="G91" s="11" t="inlineStr">
+        <is>
+          <t>₹/kL</t>
+        </is>
+      </c>
+      <c r="H91" s="11" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="I91" s="11" t="inlineStr">
+        <is>
+          <t>A 12,000-litre private tanker costs ₹1,600-1,800 in 2026, about ₹140 per kL, and up to ₹2,500 in bad weeks. That is several times the piped tariff.</t>
+        </is>
+      </c>
+      <c r="J91" s="11" t="inlineStr">
+        <is>
+          <t>₹/kL is our arithmetic: ₹1,700 ÷ 12 kL ≈ ₹142. In the 2024 crisis, 6 kL went for up to ₹3,000 (₹500/kL).</t>
+        </is>
+      </c>
+      <c r="K91" s="11" t="inlineStr">
+        <is>
+          <t>Long-term MoUs between Sanchari Cauvery and apartments (The Hindu, 2026): Private 12 kL ₹1,600-1,800, touching ₹2,500 https://www.thehindu.com/news/national/karnataka/long-term-mous-between-sanchari-cauvery-apartments-to-counter-skyrocketing-water-tanker-prices/article71278092.ece</t>
+        </is>
+      </c>
+      <c r="L91" s="11" t="inlineStr">
+        <is>
+          <t>Residents struggle to pay soaring water tanker costs (Deccan Herald, 2025): 6 kL ₹600-650; 12 kL ~₹1,400 https://www.deccanherald.com/india/karnataka/bengaluru/heat-burns-the-pocket-residents-struggle-to-pay-soaring-water-tanker-costs-3450484</t>
+        </is>
+      </c>
+      <c r="M91" s="11" t="inlineStr">
+        <is>
+          <t>Karnataka govt caps tanker water prices (New Indian Express, 2024): 2024 cap: 12 kL ₹1,000 (≤5 km) / ₹1,200 (5-10 km) https://www.newindianexpress.com/states/karnataka/2024/Mar/08/karnataka-govt-acts-caps-tanker-water-prices</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="11" t="inlineStr">
+        <is>
           <t>sanchari_rs_kl</t>
         </is>
       </c>
-      <c r="B86" s="11" t="inlineStr">
+      <c r="B92" s="11" t="inlineStr">
         <is>
           <t>Households and affordability</t>
         </is>
       </c>
-      <c r="C86" s="11" t="inlineStr">
+      <c r="C92" s="11" t="inlineStr">
         <is>
           <t>BWSSB Sanchari Cauvery tanker price</t>
         </is>
       </c>
-      <c r="D86" s="11" t="n">
+      <c r="D92" s="11" t="n">
         <v>108</v>
       </c>
-      <c r="E86" s="11" t="n">
+      <c r="E92" s="11" t="n">
         <v>107</v>
       </c>
-      <c r="F86" s="11" t="n">
+      <c r="F92" s="11" t="n">
         <v>165</v>
       </c>
-      <c r="G86" s="11" t="inlineStr">
+      <c r="G92" s="11" t="inlineStr">
         <is>
           <t>₹/kL</t>
         </is>
       </c>
-      <c r="H86" s="11" t="inlineStr">
+      <c r="H92" s="11" t="inlineStr">
         <is>
           <t>reference</t>
         </is>
       </c>
-      <c r="I86" s="11" t="inlineStr">
+      <c r="I92" s="11" t="inlineStr">
         <is>
           <t>BWSSB's own tankers sell treated Cauvery water at ₹1,290 for 12,000 litres within 2 km, about ₹108 per kL; small loads cost more per kL.</t>
         </is>
       </c>
-      <c r="J86" s="11" t="inlineStr">
+      <c r="J92" s="11" t="inlineStr">
         <is>
           <t>₹1,290 ÷ 12 = ₹107.5/kL; ₹660 ÷ 4 = ₹165/kL. Distance charges beyond 2 km add more.</t>
         </is>
       </c>
-      <c r="K86" s="11" t="inlineStr">
+      <c r="K92" s="11" t="inlineStr">
         <is>
           <t>Amidst rising water tanker prices, BWSSB launches Sanchari Cauvery (The Hindu, 2025): 4 kL ₹660; 5 kL ₹700; 6 kL ₹740; 12 kL ₹1,290 within 2 km, then +₹70/km https://www.thehindu.com/news/cities/bangalore/amidst-rising-water-tanker-prices-bwssb-launches-sanchari-cauvery-initiative/article69557670.ece</t>
         </is>
       </c>
-      <c r="L86" s="11" t="inlineStr">
+      <c r="L92" s="11" t="inlineStr">
         <is>
           <t>Sanchari Cauvery reshapes city's tanker-driven market (Bangalore Mirror, 2025): 24,743 bookings and ₹2.5 cr earned by Nov 2025 https://bangaloremirror.indiatimes.com/bangalore/civic/sanchari-cauvery-reshapes-citys-tanker-driven-market/articleshow/125667652.cms</t>
         </is>
       </c>
-      <c r="M86" s="11" t="inlineStr">
+      <c r="M92" s="11" t="inlineStr">
         <is>
           <t>Long-term MoUs between Sanchari Cauvery and apartments (The Hindu, 2026): Sanchari 12 kL about ₹1,300 vs private ₹1,600-1,800 https://www.thehindu.com/news/national/karnataka/long-term-mous-between-sanchari-cauvery-apartments-to-counter-skyrocketing-water-tanker-prices/article71278092.ece</t>
         </is>

</xml_diff>